<commit_message>
feat: update physiological datasets
</commit_message>
<xml_diff>
--- a/data/proteomics/protein_copy_statistical.xlsx
+++ b/data/proteomics/protein_copy_statistical.xlsx
@@ -8,14 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/xluhon/Documents/GitHub/De-nevo-protein-3D-structure-yeast/data/proteomics/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66AFA79F-8513-7A4E-904D-2EBB228CC5C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{522541B2-F2A4-A043-9201-445DB88D4060}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31360" yWindow="2800" windowWidth="33800" windowHeight="16480" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="26880" yWindow="0" windowWidth="40960" windowHeight="23040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlchart.v1.0" hidden="1">Sheet2!$A$2:$A$77</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">Sheet2!$J$1</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">Sheet2!$J$2:$J$77</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">Sheet2!$A$2:$A$77</definedName>
+    <definedName name="_xlchart.v1.4" hidden="1">Sheet2!$J$1</definedName>
+    <definedName name="_xlchart.v1.5" hidden="1">Sheet2!$J$2:$J$77</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -30,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="86">
   <si>
     <t>Glucose_phase(mmol/gDW)</t>
   </si>
@@ -231,6 +239,9 @@
   </si>
   <si>
     <t>Median molecules per cell_cell_system_2018</t>
+  </si>
+  <si>
+    <t>D=0.027_M</t>
   </si>
   <si>
     <t>D=0.044_M</t>
@@ -303,6 +314,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -313,7 +325,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -336,13 +348,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -437,11 +463,14 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:delete val="1"/>
+          </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Sheet2!$A$2:$A$76</c:f>
+              <c:f>Sheet2!$A$2:$A$77</c:f>
               <c:strCache>
-                <c:ptCount val="75"/>
+                <c:ptCount val="76"/>
                 <c:pt idx="0">
                   <c:v>Glucose_phase(mmol/gDW)</c:v>
                 </c:pt>
@@ -644,27 +673,30 @@
                   <c:v>Median molecules per cell_cell_system_2018</c:v>
                 </c:pt>
                 <c:pt idx="67">
+                  <c:v>D=0.027_M</c:v>
+                </c:pt>
+                <c:pt idx="68">
                   <c:v>D=0.044_M</c:v>
                 </c:pt>
-                <c:pt idx="68">
+                <c:pt idx="69">
                   <c:v>D=0.102_M</c:v>
                 </c:pt>
-                <c:pt idx="69">
+                <c:pt idx="70">
                   <c:v>D=0.152_M</c:v>
                 </c:pt>
-                <c:pt idx="70">
+                <c:pt idx="71">
                   <c:v>D=0.214_M</c:v>
                 </c:pt>
-                <c:pt idx="71">
+                <c:pt idx="72">
                   <c:v>D=0.254_M</c:v>
                 </c:pt>
-                <c:pt idx="72">
+                <c:pt idx="73">
                   <c:v>D=0.284_M</c:v>
                 </c:pt>
-                <c:pt idx="73">
+                <c:pt idx="74">
                   <c:v>D=0.334_M</c:v>
                 </c:pt>
-                <c:pt idx="74">
+                <c:pt idx="75">
                   <c:v>D=0.379_M</c:v>
                 </c:pt>
               </c:strCache>
@@ -672,10 +704,10 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet2!$J$2:$J$76</c:f>
+              <c:f>Sheet2!$J$2:$J$77</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="75"/>
+                <c:ptCount val="76"/>
                 <c:pt idx="0">
                   <c:v>120491434.23935457</c:v>
                 </c:pt>
@@ -683,7 +715,7 @@
                   <c:v>109069785.20497775</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>95199678.595657945</c:v>
+                  <c:v>95199678.595657915</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>109234782.39336768</c:v>
@@ -701,22 +733,22 @@
                   <c:v>55938194.877539828</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>59680820.010034665</c:v>
+                  <c:v>59680820.010034688</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>50281839.757225618</c:v>
+                  <c:v>50281839.757225588</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>29103726.985997025</c:v>
+                  <c:v>29103726.985997029</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>30741937.185334049</c:v>
+                  <c:v>30741937.185334053</c:v>
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>40511484.800974123</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>44021613.938357167</c:v>
+                  <c:v>44021613.938357197</c:v>
                 </c:pt>
                 <c:pt idx="14">
                   <c:v>37656800.267108344</c:v>
@@ -731,7 +763,7 @@
                   <c:v>40523307.971501589</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>40895138.240306951</c:v>
+                  <c:v>40895138.240306981</c:v>
                 </c:pt>
                 <c:pt idx="19">
                   <c:v>69133667.440792367</c:v>
@@ -740,7 +772,7 @@
                   <c:v>69270203.302799389</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>65467026.170489818</c:v>
+                  <c:v>65467026.170489848</c:v>
                 </c:pt>
                 <c:pt idx="22">
                   <c:v>85960677.000497177</c:v>
@@ -749,7 +781,7 @@
                   <c:v>90724154.877972871</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>90473101.745771378</c:v>
+                  <c:v>90473101.745771348</c:v>
                 </c:pt>
                 <c:pt idx="25">
                   <c:v>77664012.054039761</c:v>
@@ -761,7 +793,7 @@
                   <c:v>96399918.157397464</c:v>
                 </c:pt>
                 <c:pt idx="28">
-                  <c:v>74185618.030865893</c:v>
+                  <c:v>74185618.030865863</c:v>
                 </c:pt>
                 <c:pt idx="29">
                   <c:v>43774888.915245153</c:v>
@@ -785,7 +817,7 @@
                   <c:v>73418141.920373529</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>63061012.817656092</c:v>
+                  <c:v>63061012.81765607</c:v>
                 </c:pt>
                 <c:pt idx="37">
                   <c:v>59426960.766248941</c:v>
@@ -797,7 +829,7 @@
                   <c:v>56425855.057120971</c:v>
                 </c:pt>
                 <c:pt idx="40">
-                  <c:v>46825364.889163524</c:v>
+                  <c:v>46825364.889163554</c:v>
                 </c:pt>
                 <c:pt idx="41">
                   <c:v>61138905.356173508</c:v>
@@ -830,7 +862,7 @@
                   <c:v>104496016.95936453</c:v>
                 </c:pt>
                 <c:pt idx="51">
-                  <c:v>125186883.7416914</c:v>
+                  <c:v>125186883.74169138</c:v>
                 </c:pt>
                 <c:pt idx="52">
                   <c:v>79138681.737158611</c:v>
@@ -875,30 +907,33 @@
                   <c:v>61393284.855691567</c:v>
                 </c:pt>
                 <c:pt idx="66">
-                  <c:v>41856234.714812383</c:v>
+                  <c:v>41856234.714812376</c:v>
                 </c:pt>
                 <c:pt idx="67">
+                  <c:v>74298642.924967915</c:v>
+                </c:pt>
+                <c:pt idx="68">
                   <c:v>76413204.517946944</c:v>
                 </c:pt>
-                <c:pt idx="68">
+                <c:pt idx="69">
                   <c:v>84034657.500658303</c:v>
                 </c:pt>
-                <c:pt idx="69">
+                <c:pt idx="70">
                   <c:v>92066218.018570125</c:v>
                 </c:pt>
-                <c:pt idx="70">
+                <c:pt idx="71">
                   <c:v>68196502.417677805</c:v>
                 </c:pt>
-                <c:pt idx="71">
+                <c:pt idx="72">
                   <c:v>78863393.141758993</c:v>
                 </c:pt>
-                <c:pt idx="72">
+                <c:pt idx="73">
                   <c:v>81219644.018440679</c:v>
                 </c:pt>
-                <c:pt idx="73">
+                <c:pt idx="74">
                   <c:v>84063941.090120688</c:v>
                 </c:pt>
-                <c:pt idx="74">
+                <c:pt idx="75">
                   <c:v>75740273.360052153</c:v>
                 </c:pt>
               </c:numCache>
@@ -906,25 +941,25 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-38EF-4D4D-A92A-382610BCCA1A}"/>
+              <c16:uniqueId val="{00000000-EB0A-4A47-8D11-394D82332E36}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:dLbls>
+          <c:dLblPos val="ctr"/>
           <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
+          <c:showVal val="1"/>
           <c:showCatName val="0"/>
           <c:showSerName val="0"/>
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="219"/>
-        <c:overlap val="-27"/>
-        <c:axId val="2016238383"/>
-        <c:axId val="2016240031"/>
+        <c:axId val="1593236735"/>
+        <c:axId val="1593238383"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="2016238383"/>
+        <c:axId val="1593236735"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -967,7 +1002,7 @@
             <a:endParaRPr lang="en-SE"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2016240031"/>
+        <c:crossAx val="1593238383"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -975,7 +1010,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="2016240031"/>
+        <c:axId val="1593238383"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1026,7 +1061,7 @@
             <a:endParaRPr lang="en-SE"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2016238383"/>
+        <c:crossAx val="1593236735"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1123,7 +1158,7 @@
 </file>
 
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="227">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
@@ -1231,6 +1266,11 @@
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
   </cs:dataPoint>
   <cs:dataPoint3D>
     <cs:lnRef idx="0"/>
@@ -1241,6 +1281,11 @@
     <cs:fontRef idx="minor">
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
   </cs:dataPoint3D>
   <cs:dataPointLine>
     <cs:lnRef idx="0">
@@ -1272,6 +1317,9 @@
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
       <a:ln w="9525">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1629,23 +1677,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>419100</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1447800</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>22</xdr:col>
-      <xdr:colOff>635000</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>12700</xdr:rowOff>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>774700</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{717B86D6-CBF7-7240-BB77-36D4645E4658}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AC4A1545-FFA3-E74C-B914-8BC9E041C88B}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1951,10 +1999,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BX9"/>
+  <dimension ref="A1:BY9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:76" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:77" x14ac:dyDescent="0.2">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2180,10 +2228,13 @@
       <c r="BX1" s="1" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="2" spans="1:76" x14ac:dyDescent="0.2">
+      <c r="BY1" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:77" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B2">
         <v>3801</v>
@@ -2387,33 +2438,36 @@
         <v>5391</v>
       </c>
       <c r="BQ2">
+        <v>2556</v>
+      </c>
+      <c r="BR2">
         <v>2520</v>
       </c>
-      <c r="BR2">
+      <c r="BS2">
         <v>2507</v>
       </c>
-      <c r="BS2">
+      <c r="BT2">
         <v>2464</v>
       </c>
-      <c r="BT2">
+      <c r="BU2">
         <v>2485</v>
       </c>
-      <c r="BU2">
+      <c r="BV2">
         <v>2468</v>
       </c>
-      <c r="BV2">
+      <c r="BW2">
         <v>2521</v>
       </c>
-      <c r="BW2">
+      <c r="BX2">
         <v>2433</v>
       </c>
-      <c r="BX2">
+      <c r="BY2">
         <v>2416</v>
       </c>
     </row>
-    <row r="3" spans="1:76" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:77" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B3">
         <v>31699.93008138768</v>
@@ -2422,7 +2476,7 @@
         <v>28687.476382161429</v>
       </c>
       <c r="D3">
-        <v>25039.368383918449</v>
+        <v>25039.368383918441</v>
       </c>
       <c r="E3">
         <v>27809.26232010379</v>
@@ -2440,22 +2494,22 @@
         <v>17888.773545743468</v>
       </c>
       <c r="J3">
-        <v>19085.647588754291</v>
+        <v>19085.647588754298</v>
       </c>
       <c r="K3">
-        <v>16079.89758785597</v>
+        <v>16079.89758785596</v>
       </c>
       <c r="L3">
-        <v>9307.2360044761826</v>
+        <v>9307.2360044761845</v>
       </c>
       <c r="M3">
-        <v>9831.1279774013583</v>
+        <v>9831.1279774013601</v>
       </c>
       <c r="N3">
         <v>12955.383690749641</v>
       </c>
       <c r="O3">
-        <v>14077.906600050261</v>
+        <v>14077.90660005027</v>
       </c>
       <c r="P3">
         <v>12042.46890537523</v>
@@ -2470,7 +2524,7 @@
         <v>12959.164685481799</v>
       </c>
       <c r="T3">
-        <v>13078.07426936583</v>
+        <v>13078.074269365839</v>
       </c>
       <c r="U3">
         <v>22108.6240616541</v>
@@ -2479,7 +2533,7 @@
         <v>22152.28759283639</v>
       </c>
       <c r="W3">
-        <v>20936.049303002819</v>
+        <v>20936.04930300283</v>
       </c>
       <c r="X3">
         <v>27489.82315334096</v>
@@ -2488,7 +2542,7 @@
         <v>29013.16113782311</v>
       </c>
       <c r="Z3">
-        <v>28932.875518315119</v>
+        <v>28932.875518315112</v>
       </c>
       <c r="AA3">
         <v>24836.588440690681</v>
@@ -2500,7 +2554,7 @@
         <v>30828.243734377189</v>
       </c>
       <c r="AD3">
-        <v>23724.214272742531</v>
+        <v>23724.21427274252</v>
       </c>
       <c r="AE3">
         <v>13999.005089621091</v>
@@ -2524,7 +2578,7 @@
         <v>23478.778995962111</v>
       </c>
       <c r="AL3">
-        <v>20166.617466471409</v>
+        <v>20166.617466471402</v>
       </c>
       <c r="AM3">
         <v>19004.464587863429</v>
@@ -2536,7 +2590,7 @@
         <v>18044.724994282369</v>
       </c>
       <c r="AP3">
-        <v>14974.533063371769</v>
+        <v>14974.53306337178</v>
       </c>
       <c r="AQ3">
         <v>19551.936474631759</v>
@@ -2569,7 +2623,7 @@
         <v>28318.703783025619</v>
       </c>
       <c r="BA3">
-        <v>47527.290714385497</v>
+        <v>47527.29071438549</v>
       </c>
       <c r="BB3">
         <v>30113.653629055789</v>
@@ -2614,36 +2668,39 @@
         <v>11388.107003467179</v>
       </c>
       <c r="BP3">
-        <v>7764.0947347082883</v>
+        <v>7764.0947347082874</v>
       </c>
       <c r="BQ3">
+        <v>29068.326652960841</v>
+      </c>
+      <c r="BR3">
         <v>30322.7002055345</v>
       </c>
-      <c r="BR3">
+      <c r="BS3">
         <v>33520.006980717313</v>
       </c>
-      <c r="BS3">
+      <c r="BT3">
         <v>37364.536533510603</v>
       </c>
-      <c r="BT3">
+      <c r="BU3">
         <v>27443.260530252639</v>
       </c>
-      <c r="BU3">
+      <c r="BV3">
         <v>31954.37323410008</v>
       </c>
-      <c r="BV3">
+      <c r="BW3">
         <v>32217.232851424309</v>
       </c>
-      <c r="BW3">
+      <c r="BX3">
         <v>34551.558195692844</v>
       </c>
-      <c r="BX3">
+      <c r="BY3">
         <v>31349.45089406132</v>
       </c>
     </row>
-    <row r="4" spans="1:76" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:77" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B4">
         <v>248305.7799069178</v>
@@ -2676,7 +2733,7 @@
         <v>96388.775517273694</v>
       </c>
       <c r="L4">
-        <v>51497.44346481315</v>
+        <v>51497.443464813157</v>
       </c>
       <c r="M4">
         <v>53751.599616567422</v>
@@ -2685,7 +2742,7 @@
         <v>68179.03059273884</v>
       </c>
       <c r="O4">
-        <v>71730.571303751552</v>
+        <v>71730.571303751567</v>
       </c>
       <c r="P4">
         <v>63910.569457566991</v>
@@ -2766,13 +2823,13 @@
         <v>89473.927213093062</v>
       </c>
       <c r="AP4">
-        <v>82237.749540781166</v>
+        <v>82237.749540781151</v>
       </c>
       <c r="AQ4">
         <v>113134.1287620463</v>
       </c>
       <c r="AR4">
-        <v>90434.901848091366</v>
+        <v>90434.90184809138</v>
       </c>
       <c r="AS4">
         <v>118737.5902741415</v>
@@ -2847,33 +2904,36 @@
         <v>27505.07111669971</v>
       </c>
       <c r="BQ4">
+        <v>120732.9908766626</v>
+      </c>
+      <c r="BR4">
         <v>116672.5530703134</v>
       </c>
-      <c r="BR4">
+      <c r="BS4">
         <v>101701.58965527589</v>
       </c>
-      <c r="BS4">
+      <c r="BT4">
         <v>103453.4782046555</v>
       </c>
-      <c r="BT4">
+      <c r="BU4">
         <v>73029.995712406468</v>
       </c>
-      <c r="BU4">
-        <v>85832.681393492283</v>
-      </c>
       <c r="BV4">
+        <v>85832.681393492298</v>
+      </c>
+      <c r="BW4">
         <v>86498.885958305895</v>
       </c>
-      <c r="BW4">
+      <c r="BX4">
         <v>92359.273897153471</v>
       </c>
-      <c r="BX4">
+      <c r="BY4">
         <v>84989.720816127578</v>
       </c>
     </row>
-    <row r="5" spans="1:76" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:77" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B5">
         <v>0.33315246856710917</v>
@@ -3077,33 +3137,36 @@
         <v>3.3597834780000002</v>
       </c>
       <c r="BQ5">
+        <v>7.8118557164171198</v>
+      </c>
+      <c r="BR5">
         <v>15.458391645546151</v>
       </c>
-      <c r="BR5">
+      <c r="BS5">
         <v>6.0572404505728503</v>
       </c>
-      <c r="BS5">
+      <c r="BT5">
         <v>9.9360493440266104</v>
       </c>
-      <c r="BT5">
+      <c r="BU5">
         <v>7.4029580526572403</v>
       </c>
-      <c r="BU5">
+      <c r="BV5">
         <v>12.9261462771642</v>
       </c>
-      <c r="BV5">
+      <c r="BW5">
         <v>7.3988993561487701</v>
       </c>
-      <c r="BW5">
+      <c r="BX5">
         <v>10.692399393006699</v>
       </c>
-      <c r="BX5">
+      <c r="BY5">
         <v>10.408059734663</v>
       </c>
     </row>
-    <row r="6" spans="1:76" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:77" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B6">
         <v>167.96897045455651</v>
@@ -3307,33 +3370,36 @@
         <v>1391.58692875209</v>
       </c>
       <c r="BQ6">
+        <v>1256.5757238989299</v>
+      </c>
+      <c r="BR6">
         <v>1379.6400087600821</v>
       </c>
-      <c r="BR6">
+      <c r="BS6">
         <v>1670.3116732609601</v>
       </c>
-      <c r="BS6">
+      <c r="BT6">
         <v>1896.1662587157541</v>
       </c>
-      <c r="BT6">
+      <c r="BU6">
         <v>1386.5880154895669</v>
       </c>
-      <c r="BU6">
+      <c r="BV6">
         <v>1552.23531400505</v>
       </c>
-      <c r="BV6">
+      <c r="BW6">
         <v>1468.786393033914</v>
       </c>
-      <c r="BW6">
+      <c r="BX6">
         <v>1615.8124859845971</v>
       </c>
-      <c r="BX6">
+      <c r="BY6">
         <v>1438.2178947730779</v>
       </c>
     </row>
-    <row r="7" spans="1:76" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:77" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B7">
         <v>712.2876501272201</v>
@@ -3537,33 +3603,36 @@
         <v>2621.8133906241101</v>
       </c>
       <c r="BQ7">
+        <v>3878.485182046827</v>
+      </c>
+      <c r="BR7">
         <v>4146.8476327401168</v>
       </c>
-      <c r="BR7">
+      <c r="BS7">
         <v>5222.1472043664371</v>
       </c>
-      <c r="BS7">
+      <c r="BT7">
         <v>6016.9140901092924</v>
       </c>
-      <c r="BT7">
+      <c r="BU7">
         <v>4393.5288895098929</v>
       </c>
-      <c r="BU7">
+      <c r="BV7">
         <v>4919.7547846049674</v>
       </c>
-      <c r="BV7">
+      <c r="BW7">
         <v>4680.7079662738352</v>
       </c>
-      <c r="BW7">
+      <c r="BX7">
         <v>4969.8417109000629</v>
       </c>
-      <c r="BX7">
+      <c r="BY7">
         <v>4556.437668683825</v>
       </c>
     </row>
-    <row r="8" spans="1:76" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:77" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B8">
         <v>3466.373731147874</v>
@@ -3767,33 +3836,36 @@
         <v>5354.31353239906</v>
       </c>
       <c r="BQ8">
+        <v>17772.448533641262</v>
+      </c>
+      <c r="BR8">
         <v>18106.018183062781</v>
       </c>
-      <c r="BR8">
+      <c r="BS8">
         <v>21049.81994745378</v>
       </c>
-      <c r="BS8">
+      <c r="BT8">
         <v>23773.5869697374</v>
       </c>
-      <c r="BT8">
+      <c r="BU8">
         <v>17268.17173946237</v>
       </c>
-      <c r="BU8">
+      <c r="BV8">
         <v>19295.91794866593</v>
       </c>
-      <c r="BV8">
+      <c r="BW8">
         <v>18321.802293552231</v>
       </c>
-      <c r="BW8">
+      <c r="BX8">
         <v>19259.213713720699</v>
       </c>
-      <c r="BX8">
+      <c r="BY8">
         <v>17393.997536666859</v>
       </c>
     </row>
-    <row r="9" spans="1:76" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:77" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B9">
         <v>8122726.5924343634</v>
@@ -3997,27 +4069,30 @@
         <v>746357.568074079</v>
       </c>
       <c r="BQ9">
+        <v>3989325.6406153799</v>
+      </c>
+      <c r="BR9">
         <v>3563066.2821484101</v>
       </c>
-      <c r="BR9">
+      <c r="BS9">
         <v>2186908.8085103841</v>
       </c>
-      <c r="BS9">
+      <c r="BT9">
         <v>1526611.414481163</v>
       </c>
-      <c r="BT9">
+      <c r="BU9">
         <v>1197000.573967651</v>
       </c>
-      <c r="BU9">
+      <c r="BV9">
         <v>1459414.0661639229</v>
       </c>
-      <c r="BV9">
+      <c r="BW9">
         <v>1515763.9115661869</v>
       </c>
-      <c r="BW9">
+      <c r="BX9">
         <v>1527797.363900427</v>
       </c>
-      <c r="BX9">
+      <c r="BY9">
         <v>1382972.910274663</v>
       </c>
     </row>
@@ -4027,44 +4102,47 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5681073C-E082-7E4B-93CB-BF438F127318}">
-  <dimension ref="A1:J76"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFBC6659-2F17-4240-A8B7-39F0E1000ACE}">
+  <dimension ref="A1:J77"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="32" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="J1" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B1" t="s">
-        <v>75</v>
-      </c>
-      <c r="C1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D1" t="s">
-        <v>77</v>
-      </c>
-      <c r="E1" t="s">
-        <v>78</v>
-      </c>
-      <c r="F1" t="s">
-        <v>79</v>
-      </c>
-      <c r="G1" t="s">
-        <v>80</v>
-      </c>
-      <c r="H1" t="s">
-        <v>81</v>
-      </c>
-      <c r="I1" t="s">
-        <v>82</v>
-      </c>
-      <c r="J1" t="s">
-        <v>83</v>
-      </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2">
@@ -4097,7 +4175,7 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B3">
@@ -4130,14 +4208,14 @@
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B4">
         <v>3802</v>
       </c>
       <c r="C4">
-        <v>25039.368383918449</v>
+        <v>25039.368383918441</v>
       </c>
       <c r="D4">
         <v>154715.8728319417</v>
@@ -4159,11 +4237,11 @@
       </c>
       <c r="J4">
         <f t="shared" si="0"/>
-        <v>95199678.595657945</v>
+        <v>95199678.595657915</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B5">
@@ -4196,7 +4274,7 @@
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B6">
@@ -4229,7 +4307,7 @@
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B7">
@@ -4262,7 +4340,7 @@
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B8">
@@ -4295,7 +4373,7 @@
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+      <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B9">
@@ -4328,14 +4406,14 @@
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+      <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B10">
         <v>3127</v>
       </c>
       <c r="C10">
-        <v>19085.647588754291</v>
+        <v>19085.647588754298</v>
       </c>
       <c r="D10">
         <v>123933.3220014994</v>
@@ -4357,18 +4435,18 @@
       </c>
       <c r="J10">
         <f t="shared" si="0"/>
-        <v>59680820.010034665</v>
+        <v>59680820.010034688</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+      <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B11">
         <v>3127</v>
       </c>
       <c r="C11">
-        <v>16079.89758785597</v>
+        <v>16079.89758785596</v>
       </c>
       <c r="D11">
         <v>96388.775517273694</v>
@@ -4390,21 +4468,21 @@
       </c>
       <c r="J11">
         <f t="shared" si="0"/>
-        <v>50281839.757225618</v>
+        <v>50281839.757225588</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+      <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B12">
         <v>3127</v>
       </c>
       <c r="C12">
-        <v>9307.2360044761826</v>
+        <v>9307.2360044761845</v>
       </c>
       <c r="D12">
-        <v>51497.44346481315</v>
+        <v>51497.443464813157</v>
       </c>
       <c r="E12">
         <v>0</v>
@@ -4423,18 +4501,18 @@
       </c>
       <c r="J12">
         <f t="shared" si="0"/>
-        <v>29103726.985997025</v>
+        <v>29103726.985997029</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
+      <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B13">
         <v>3127</v>
       </c>
       <c r="C13">
-        <v>9831.1279774013583</v>
+        <v>9831.1279774013601</v>
       </c>
       <c r="D13">
         <v>53751.599616567422</v>
@@ -4456,11 +4534,11 @@
       </c>
       <c r="J13">
         <f t="shared" si="0"/>
-        <v>30741937.185334049</v>
+        <v>30741937.185334053</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
+      <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B14">
@@ -4493,17 +4571,17 @@
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
+      <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B15">
         <v>3127</v>
       </c>
       <c r="C15">
-        <v>14077.906600050261</v>
+        <v>14077.90660005027</v>
       </c>
       <c r="D15">
-        <v>71730.571303751552</v>
+        <v>71730.571303751567</v>
       </c>
       <c r="E15">
         <v>0</v>
@@ -4522,11 +4600,11 @@
       </c>
       <c r="J15">
         <f t="shared" si="0"/>
-        <v>44021613.938357167</v>
+        <v>44021613.938357197</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
+      <c r="A16" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B16">
@@ -4559,7 +4637,7 @@
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+      <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B17">
@@ -4592,7 +4670,7 @@
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
+      <c r="A18" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B18">
@@ -4625,7 +4703,7 @@
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
+      <c r="A19" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B19">
@@ -4658,14 +4736,14 @@
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
+      <c r="A20" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B20">
         <v>3127</v>
       </c>
       <c r="C20">
-        <v>13078.07426936583</v>
+        <v>13078.074269365839</v>
       </c>
       <c r="D20">
         <v>68304.716232255683</v>
@@ -4687,11 +4765,11 @@
       </c>
       <c r="J20">
         <f t="shared" si="0"/>
-        <v>40895138.240306951</v>
+        <v>40895138.240306981</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+      <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
       <c r="B21">
@@ -4724,7 +4802,7 @@
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
+      <c r="A22" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B22">
@@ -4757,14 +4835,14 @@
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
+      <c r="A23" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B23">
         <v>3127</v>
       </c>
       <c r="C23">
-        <v>20936.049303002819</v>
+        <v>20936.04930300283</v>
       </c>
       <c r="D23">
         <v>106894.8860790297</v>
@@ -4786,11 +4864,11 @@
       </c>
       <c r="J23">
         <f t="shared" si="0"/>
-        <v>65467026.170489818</v>
+        <v>65467026.170489848</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
+      <c r="A24" s="1" t="s">
         <v>22</v>
       </c>
       <c r="B24">
@@ -4823,7 +4901,7 @@
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
+      <c r="A25" s="1" t="s">
         <v>23</v>
       </c>
       <c r="B25">
@@ -4856,14 +4934,14 @@
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
+      <c r="A26" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B26">
         <v>3127</v>
       </c>
       <c r="C26">
-        <v>28932.875518315119</v>
+        <v>28932.875518315112</v>
       </c>
       <c r="D26">
         <v>149600.8276335788</v>
@@ -4885,11 +4963,11 @@
       </c>
       <c r="J26">
         <f t="shared" si="0"/>
-        <v>90473101.745771378</v>
+        <v>90473101.745771348</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
+      <c r="A27" s="1" t="s">
         <v>25</v>
       </c>
       <c r="B27">
@@ -4922,7 +5000,7 @@
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
+      <c r="A28" s="1" t="s">
         <v>26</v>
       </c>
       <c r="B28">
@@ -4955,7 +5033,7 @@
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
+      <c r="A29" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B29">
@@ -4988,14 +5066,14 @@
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
+      <c r="A30" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B30">
         <v>3127</v>
       </c>
       <c r="C30">
-        <v>23724.214272742531</v>
+        <v>23724.21427274252</v>
       </c>
       <c r="D30">
         <v>134114.44931428449</v>
@@ -5017,11 +5095,11 @@
       </c>
       <c r="J30">
         <f t="shared" si="0"/>
-        <v>74185618.030865893</v>
+        <v>74185618.030865863</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
+      <c r="A31" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B31">
@@ -5054,7 +5132,7 @@
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
+      <c r="A32" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B32">
@@ -5087,7 +5165,7 @@
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
+      <c r="A33" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B33">
@@ -5120,7 +5198,7 @@
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
+      <c r="A34" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B34">
@@ -5153,7 +5231,7 @@
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
+      <c r="A35" s="1" t="s">
         <v>33</v>
       </c>
       <c r="B35">
@@ -5186,7 +5264,7 @@
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
+      <c r="A36" s="1" t="s">
         <v>34</v>
       </c>
       <c r="B36">
@@ -5219,7 +5297,7 @@
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A37" t="s">
+      <c r="A37" s="1" t="s">
         <v>35</v>
       </c>
       <c r="B37">
@@ -5252,14 +5330,14 @@
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
+      <c r="A38" s="1" t="s">
         <v>36</v>
       </c>
       <c r="B38">
         <v>3127</v>
       </c>
       <c r="C38">
-        <v>20166.617466471409</v>
+        <v>20166.617466471402</v>
       </c>
       <c r="D38">
         <v>109564.778723442</v>
@@ -5281,11 +5359,11 @@
       </c>
       <c r="J38">
         <f t="shared" si="0"/>
-        <v>63061012.817656092</v>
+        <v>63061012.81765607</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A39" t="s">
+      <c r="A39" s="1" t="s">
         <v>37</v>
       </c>
       <c r="B39">
@@ -5318,7 +5396,7 @@
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
+      <c r="A40" s="1" t="s">
         <v>38</v>
       </c>
       <c r="B40">
@@ -5351,7 +5429,7 @@
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
+      <c r="A41" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B41">
@@ -5384,17 +5462,17 @@
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A42" t="s">
+      <c r="A42" s="1" t="s">
         <v>40</v>
       </c>
       <c r="B42">
         <v>3127</v>
       </c>
       <c r="C42">
-        <v>14974.533063371769</v>
+        <v>14974.53306337178</v>
       </c>
       <c r="D42">
-        <v>82237.749540781166</v>
+        <v>82237.749540781151</v>
       </c>
       <c r="E42">
         <v>0</v>
@@ -5413,11 +5491,11 @@
       </c>
       <c r="J42">
         <f t="shared" si="0"/>
-        <v>46825364.889163524</v>
+        <v>46825364.889163554</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
+      <c r="A43" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B43">
@@ -5450,7 +5528,7 @@
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
+      <c r="A44" s="1" t="s">
         <v>42</v>
       </c>
       <c r="B44">
@@ -5460,7 +5538,7 @@
         <v>16678.348440522412</v>
       </c>
       <c r="D44">
-        <v>90434.901848091366</v>
+        <v>90434.90184809138</v>
       </c>
       <c r="E44">
         <v>0</v>
@@ -5483,7 +5561,7 @@
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
+      <c r="A45" s="1" t="s">
         <v>43</v>
       </c>
       <c r="B45">
@@ -5516,7 +5594,7 @@
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
+      <c r="A46" s="1" t="s">
         <v>44</v>
       </c>
       <c r="B46">
@@ -5549,7 +5627,7 @@
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
+      <c r="A47" s="1" t="s">
         <v>45</v>
       </c>
       <c r="B47">
@@ -5582,7 +5660,7 @@
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
+      <c r="A48" s="1" t="s">
         <v>46</v>
       </c>
       <c r="B48">
@@ -5615,7 +5693,7 @@
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
+      <c r="A49" s="1" t="s">
         <v>47</v>
       </c>
       <c r="B49">
@@ -5648,7 +5726,7 @@
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
+      <c r="A50" s="1" t="s">
         <v>48</v>
       </c>
       <c r="B50">
@@ -5681,7 +5759,7 @@
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
+      <c r="A51" s="1" t="s">
         <v>49</v>
       </c>
       <c r="B51">
@@ -5714,7 +5792,7 @@
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
+      <c r="A52" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B52">
@@ -5747,14 +5825,14 @@
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
+      <c r="A53" s="1" t="s">
         <v>51</v>
       </c>
       <c r="B53">
         <v>2634</v>
       </c>
       <c r="C53">
-        <v>47527.290714385497</v>
+        <v>47527.29071438549</v>
       </c>
       <c r="D53">
         <v>194937.71464623071</v>
@@ -5776,11 +5854,11 @@
       </c>
       <c r="J53">
         <f t="shared" si="0"/>
-        <v>125186883.7416914</v>
+        <v>125186883.74169138</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A54" t="s">
+      <c r="A54" s="1" t="s">
         <v>52</v>
       </c>
       <c r="B54">
@@ -5813,7 +5891,7 @@
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A55" t="s">
+      <c r="A55" s="1" t="s">
         <v>53</v>
       </c>
       <c r="B55">
@@ -5846,7 +5924,7 @@
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A56" t="s">
+      <c r="A56" s="1" t="s">
         <v>54</v>
       </c>
       <c r="B56">
@@ -5879,7 +5957,7 @@
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A57" t="s">
+      <c r="A57" s="1" t="s">
         <v>55</v>
       </c>
       <c r="B57">
@@ -5912,7 +5990,7 @@
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A58" t="s">
+      <c r="A58" s="1" t="s">
         <v>56</v>
       </c>
       <c r="B58">
@@ -5945,7 +6023,7 @@
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A59" t="s">
+      <c r="A59" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B59">
@@ -5978,7 +6056,7 @@
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A60" t="s">
+      <c r="A60" s="1" t="s">
         <v>58</v>
       </c>
       <c r="B60">
@@ -6011,7 +6089,7 @@
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A61" t="s">
+      <c r="A61" s="1" t="s">
         <v>59</v>
       </c>
       <c r="B61">
@@ -6044,7 +6122,7 @@
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A62" t="s">
+      <c r="A62" s="1" t="s">
         <v>60</v>
       </c>
       <c r="B62">
@@ -6077,7 +6155,7 @@
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A63" t="s">
+      <c r="A63" s="1" t="s">
         <v>61</v>
       </c>
       <c r="B63">
@@ -6110,7 +6188,7 @@
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A64" t="s">
+      <c r="A64" s="1" t="s">
         <v>62</v>
       </c>
       <c r="B64">
@@ -6143,7 +6221,7 @@
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A65" t="s">
+      <c r="A65" s="1" t="s">
         <v>63</v>
       </c>
       <c r="B65">
@@ -6176,7 +6254,7 @@
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A66" t="s">
+      <c r="A66" s="1" t="s">
         <v>64</v>
       </c>
       <c r="B66">
@@ -6209,7 +6287,7 @@
       </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A67" t="s">
+      <c r="A67" s="1" t="s">
         <v>65</v>
       </c>
       <c r="B67">
@@ -6237,19 +6315,19 @@
         <v>1392598.8002863601</v>
       </c>
       <c r="J67">
-        <f t="shared" ref="J67:J76" si="1">B67*C67</f>
+        <f t="shared" ref="J67:J77" si="1">B67*C67</f>
         <v>61393284.855691567</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A68" t="s">
+      <c r="A68" s="1" t="s">
         <v>66</v>
       </c>
       <c r="B68">
         <v>5391</v>
       </c>
       <c r="C68">
-        <v>7764.0947347082883</v>
+        <v>7764.0947347082874</v>
       </c>
       <c r="D68">
         <v>27505.07111669971</v>
@@ -6271,269 +6349,302 @@
       </c>
       <c r="J68">
         <f t="shared" si="1"/>
-        <v>41856234.714812383</v>
+        <v>41856234.714812376</v>
       </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A69" t="s">
+      <c r="A69" s="1" t="s">
         <v>67</v>
       </c>
       <c r="B69">
-        <v>2520</v>
+        <v>2556</v>
       </c>
       <c r="C69">
-        <v>30322.7002055345</v>
+        <v>29068.326652960841</v>
       </c>
       <c r="D69">
-        <v>116672.5530703134</v>
+        <v>120732.9908766626</v>
       </c>
       <c r="E69">
-        <v>15.458391645546151</v>
+        <v>7.8118557164171198</v>
       </c>
       <c r="F69">
-        <v>1379.6400087600821</v>
+        <v>1256.5757238989299</v>
       </c>
       <c r="G69">
-        <v>4146.8476327401168</v>
+        <v>3878.485182046827</v>
       </c>
       <c r="H69">
-        <v>18106.018183062781</v>
+        <v>17772.448533641262</v>
       </c>
       <c r="I69">
-        <v>3563066.2821484101</v>
+        <v>3989325.6406153799</v>
       </c>
       <c r="J69">
         <f t="shared" si="1"/>
-        <v>76413204.517946944</v>
+        <v>74298642.924967915</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A70" t="s">
+      <c r="A70" s="1" t="s">
         <v>68</v>
       </c>
       <c r="B70">
-        <v>2507</v>
+        <v>2520</v>
       </c>
       <c r="C70">
-        <v>33520.006980717313</v>
+        <v>30322.7002055345</v>
       </c>
       <c r="D70">
-        <v>101701.58965527589</v>
+        <v>116672.5530703134</v>
       </c>
       <c r="E70">
-        <v>6.0572404505728503</v>
+        <v>15.458391645546151</v>
       </c>
       <c r="F70">
-        <v>1670.3116732609601</v>
+        <v>1379.6400087600821</v>
       </c>
       <c r="G70">
-        <v>5222.1472043664371</v>
+        <v>4146.8476327401168</v>
       </c>
       <c r="H70">
-        <v>21049.81994745378</v>
+        <v>18106.018183062781</v>
       </c>
       <c r="I70">
-        <v>2186908.8085103841</v>
+        <v>3563066.2821484101</v>
       </c>
       <c r="J70">
         <f t="shared" si="1"/>
-        <v>84034657.500658303</v>
+        <v>76413204.517946944</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A71" t="s">
+      <c r="A71" s="1" t="s">
         <v>69</v>
       </c>
       <c r="B71">
-        <v>2464</v>
+        <v>2507</v>
       </c>
       <c r="C71">
-        <v>37364.536533510603</v>
+        <v>33520.006980717313</v>
       </c>
       <c r="D71">
-        <v>103453.4782046555</v>
+        <v>101701.58965527589</v>
       </c>
       <c r="E71">
-        <v>9.9360493440266104</v>
+        <v>6.0572404505728503</v>
       </c>
       <c r="F71">
-        <v>1896.1662587157541</v>
+        <v>1670.3116732609601</v>
       </c>
       <c r="G71">
-        <v>6016.9140901092924</v>
+        <v>5222.1472043664371</v>
       </c>
       <c r="H71">
-        <v>23773.5869697374</v>
+        <v>21049.81994745378</v>
       </c>
       <c r="I71">
-        <v>1526611.414481163</v>
+        <v>2186908.8085103841</v>
       </c>
       <c r="J71">
         <f t="shared" si="1"/>
-        <v>92066218.018570125</v>
+        <v>84034657.500658303</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A72" t="s">
+      <c r="A72" s="1" t="s">
         <v>70</v>
       </c>
       <c r="B72">
-        <v>2485</v>
+        <v>2464</v>
       </c>
       <c r="C72">
-        <v>27443.260530252639</v>
+        <v>37364.536533510603</v>
       </c>
       <c r="D72">
-        <v>73029.995712406468</v>
+        <v>103453.4782046555</v>
       </c>
       <c r="E72">
-        <v>7.4029580526572403</v>
+        <v>9.9360493440266104</v>
       </c>
       <c r="F72">
-        <v>1386.5880154895669</v>
+        <v>1896.1662587157541</v>
       </c>
       <c r="G72">
-        <v>4393.5288895098929</v>
+        <v>6016.9140901092924</v>
       </c>
       <c r="H72">
-        <v>17268.17173946237</v>
+        <v>23773.5869697374</v>
       </c>
       <c r="I72">
-        <v>1197000.573967651</v>
+        <v>1526611.414481163</v>
       </c>
       <c r="J72">
         <f t="shared" si="1"/>
-        <v>68196502.417677805</v>
+        <v>92066218.018570125</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A73" t="s">
+      <c r="A73" s="1" t="s">
         <v>71</v>
       </c>
       <c r="B73">
-        <v>2468</v>
+        <v>2485</v>
       </c>
       <c r="C73">
-        <v>31954.37323410008</v>
+        <v>27443.260530252639</v>
       </c>
       <c r="D73">
-        <v>85832.681393492283</v>
+        <v>73029.995712406468</v>
       </c>
       <c r="E73">
-        <v>12.9261462771642</v>
+        <v>7.4029580526572403</v>
       </c>
       <c r="F73">
-        <v>1552.23531400505</v>
+        <v>1386.5880154895669</v>
       </c>
       <c r="G73">
-        <v>4919.7547846049674</v>
+        <v>4393.5288895098929</v>
       </c>
       <c r="H73">
-        <v>19295.91794866593</v>
+        <v>17268.17173946237</v>
       </c>
       <c r="I73">
-        <v>1459414.0661639229</v>
+        <v>1197000.573967651</v>
       </c>
       <c r="J73">
         <f t="shared" si="1"/>
-        <v>78863393.141758993</v>
+        <v>68196502.417677805</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A74" t="s">
+      <c r="A74" s="1" t="s">
         <v>72</v>
       </c>
       <c r="B74">
-        <v>2521</v>
+        <v>2468</v>
       </c>
       <c r="C74">
-        <v>32217.232851424309</v>
+        <v>31954.37323410008</v>
       </c>
       <c r="D74">
-        <v>86498.885958305895</v>
+        <v>85832.681393492298</v>
       </c>
       <c r="E74">
-        <v>7.3988993561487701</v>
+        <v>12.9261462771642</v>
       </c>
       <c r="F74">
-        <v>1468.786393033914</v>
+        <v>1552.23531400505</v>
       </c>
       <c r="G74">
-        <v>4680.7079662738352</v>
+        <v>4919.7547846049674</v>
       </c>
       <c r="H74">
-        <v>18321.802293552231</v>
+        <v>19295.91794866593</v>
       </c>
       <c r="I74">
-        <v>1515763.9115661869</v>
+        <v>1459414.0661639229</v>
       </c>
       <c r="J74">
         <f t="shared" si="1"/>
-        <v>81219644.018440679</v>
+        <v>78863393.141758993</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A75" t="s">
+      <c r="A75" s="1" t="s">
         <v>73</v>
       </c>
       <c r="B75">
-        <v>2433</v>
+        <v>2521</v>
       </c>
       <c r="C75">
-        <v>34551.558195692844</v>
+        <v>32217.232851424309</v>
       </c>
       <c r="D75">
-        <v>92359.273897153471</v>
+        <v>86498.885958305895</v>
       </c>
       <c r="E75">
-        <v>10.692399393006699</v>
+        <v>7.3988993561487701</v>
       </c>
       <c r="F75">
-        <v>1615.8124859845971</v>
+        <v>1468.786393033914</v>
       </c>
       <c r="G75">
-        <v>4969.8417109000629</v>
+        <v>4680.7079662738352</v>
       </c>
       <c r="H75">
-        <v>19259.213713720699</v>
+        <v>18321.802293552231</v>
       </c>
       <c r="I75">
-        <v>1527797.363900427</v>
+        <v>1515763.9115661869</v>
       </c>
       <c r="J75">
         <f t="shared" si="1"/>
+        <v>81219644.018440679</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A76" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B76">
+        <v>2433</v>
+      </c>
+      <c r="C76">
+        <v>34551.558195692844</v>
+      </c>
+      <c r="D76">
+        <v>92359.273897153471</v>
+      </c>
+      <c r="E76">
+        <v>10.692399393006699</v>
+      </c>
+      <c r="F76">
+        <v>1615.8124859845971</v>
+      </c>
+      <c r="G76">
+        <v>4969.8417109000629</v>
+      </c>
+      <c r="H76">
+        <v>19259.213713720699</v>
+      </c>
+      <c r="I76">
+        <v>1527797.363900427</v>
+      </c>
+      <c r="J76">
+        <f t="shared" si="1"/>
         <v>84063941.090120688</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A76" t="s">
-        <v>74</v>
-      </c>
-      <c r="B76">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A77" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B77">
         <v>2416</v>
       </c>
-      <c r="C76">
+      <c r="C77">
         <v>31349.45089406132</v>
       </c>
-      <c r="D76">
+      <c r="D77">
         <v>84989.720816127578</v>
       </c>
-      <c r="E76">
+      <c r="E77">
         <v>10.408059734663</v>
       </c>
-      <c r="F76">
+      <c r="F77">
         <v>1438.2178947730779</v>
       </c>
-      <c r="G76">
+      <c r="G77">
         <v>4556.437668683825</v>
       </c>
-      <c r="H76">
+      <c r="H77">
         <v>17393.997536666859</v>
       </c>
-      <c r="I76">
+      <c r="I77">
         <v>1382972.910274663</v>
       </c>
-      <c r="J76">
+      <c r="J77">
         <f t="shared" si="1"/>
         <v>75740273.360052153</v>
       </c>

</xml_diff>

<commit_message>
fix: refine omics analysis pipeline
</commit_message>
<xml_diff>
--- a/data/proteomics/protein_copy_statistical.xlsx
+++ b/data/proteomics/protein_copy_statistical.xlsx
@@ -1082,7 +1082,7 @@
         <v>16079.89758785596</v>
       </c>
       <c r="L3" t="n">
-        <v>9307.236004476184</v>
+        <v>9307.236004476186</v>
       </c>
       <c r="M3" t="n">
         <v>9831.12797740136</v>
@@ -1091,7 +1091,7 @@
         <v>12955.38369074964</v>
       </c>
       <c r="O3" t="n">
-        <v>14077.90660005027</v>
+        <v>14077.90660005026</v>
       </c>
       <c r="P3" t="n">
         <v>12042.46890537523</v>
@@ -1136,7 +1136,7 @@
         <v>30828.24373437719</v>
       </c>
       <c r="AD3" t="n">
-        <v>23724.21427274252</v>
+        <v>23724.21427274253</v>
       </c>
       <c r="AE3" t="n">
         <v>13999.00508962109</v>
@@ -1193,7 +1193,7 @@
         <v>26692.50099691877</v>
       </c>
       <c r="AW3" t="n">
-        <v>30739.82382791224</v>
+        <v>30739.82382791223</v>
       </c>
       <c r="AX3" t="n">
         <v>31699.64696088852</v>
@@ -1317,7 +1317,7 @@
         <v>96388.77551727369</v>
       </c>
       <c r="L4" t="n">
-        <v>51497.44346481316</v>
+        <v>51497.44346481315</v>
       </c>
       <c r="M4" t="n">
         <v>53751.59961656742</v>
@@ -1329,7 +1329,7 @@
         <v>71730.57130375157</v>
       </c>
       <c r="P4" t="n">
-        <v>63910.56945756699</v>
+        <v>63910.56945756701</v>
       </c>
       <c r="Q4" t="n">
         <v>62287.14171905869</v>
@@ -1404,7 +1404,7 @@
         <v>86462.43162682682</v>
       </c>
       <c r="AO4" t="n">
-        <v>89473.92721309306</v>
+        <v>89473.92721309305</v>
       </c>
       <c r="AP4" t="n">
         <v>82237.74954078115</v>
@@ -1413,7 +1413,7 @@
         <v>113134.1287620463</v>
       </c>
       <c r="AR4" t="n">
-        <v>90434.90184809138</v>
+        <v>90434.90184809137</v>
       </c>
       <c r="AS4" t="n">
         <v>118737.5902741415</v>
@@ -1449,7 +1449,7 @@
         <v>191407.9031324337</v>
       </c>
       <c r="BD4" t="n">
-        <v>95665.31281119703</v>
+        <v>95665.31281119701</v>
       </c>
       <c r="BE4" t="n">
         <v>137212.9599842691</v>
@@ -1760,10 +1760,10 @@
         <v>167.9689704545565</v>
       </c>
       <c r="C6" t="n">
-        <v>223.4463347942533</v>
+        <v>223.4463347942532</v>
       </c>
       <c r="D6" t="n">
-        <v>229.1642297708296</v>
+        <v>229.1642297708295</v>
       </c>
       <c r="E6" t="n">
         <v>598.8225460547256</v>
@@ -1910,7 +1910,7 @@
         <v>253.2547174155409</v>
       </c>
       <c r="BA6" t="n">
-        <v>1459.815858569298</v>
+        <v>1459.815858569299</v>
       </c>
       <c r="BB6" t="n">
         <v>1010.238493326309</v>
@@ -1931,7 +1931,7 @@
         <v>1375.226008848034</v>
       </c>
       <c r="BH6" t="n">
-        <v>1354.791949708647</v>
+        <v>1354.791949708646</v>
       </c>
       <c r="BI6" t="n">
         <v>196.8</v>
@@ -2139,16 +2139,16 @@
         <v>1165.831146022247</v>
       </c>
       <c r="AY7" t="n">
-        <v>1015.350537744355</v>
+        <v>1015.350537744354</v>
       </c>
       <c r="AZ7" t="n">
         <v>1105.483725819433</v>
       </c>
       <c r="BA7" t="n">
-        <v>4797.799119491618</v>
+        <v>4797.799119491619</v>
       </c>
       <c r="BB7" t="n">
-        <v>3234.263269472808</v>
+        <v>3234.263269472807</v>
       </c>
       <c r="BC7" t="n">
         <v>5048.577899838969</v>
@@ -2347,7 +2347,7 @@
         <v>3629.00075118834</v>
       </c>
       <c r="AP8" t="n">
-        <v>2758.22897344555</v>
+        <v>2758.228973445551</v>
       </c>
       <c r="AQ8" t="n">
         <v>3474.5808186001</v>
@@ -2392,7 +2392,7 @@
         <v>11793.3141094675</v>
       </c>
       <c r="BE8" t="n">
-        <v>16260.44543031608</v>
+        <v>16260.44543031607</v>
       </c>
       <c r="BF8" t="n">
         <v>15817.18243947031</v>
@@ -2401,7 +2401,7 @@
         <v>16555.3698080685</v>
       </c>
       <c r="BH8" t="n">
-        <v>16063.3839714719</v>
+        <v>16063.38397147189</v>
       </c>
       <c r="BI8" t="n">
         <v>5388</v>

</xml_diff>

<commit_message>
feat: add new analysis
</commit_message>
<xml_diff>
--- a/data/proteomics/protein_copy_statistical.xlsx
+++ b/data/proteomics/protein_copy_statistical.xlsx
@@ -425,48 +425,68 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>C-lim rep1 prot (fmol mgDW-1)</t>
+          <t>ref_glc_mm_rich_aerobic(mmol/gDW)_x</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>C-lim rep2 prot (fmol mgDW-1)</t>
+          <t>maltose(mmol/gDW)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>C/N=115 rep1 prot (fmol mgDW-1)</t>
+          <t>oleate(mmol/gDW)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>C/N=115 rep2 prot (fmol mgDW-1)</t>
+          <t>fructose(mmol/gDW)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>C/N=30 rep1 prot (fmol mgDW-1)</t>
+          <t>sucrose(mmol/gDW)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>C/N=30 rep2 prot (fmol mgDW-1)</t>
+          <t>trehalose(mmol/gDW)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>C/N=50 rep1 prot (fmol mgDW-1)</t>
+          <t>lactate(mmol/gDW)</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>C/N=50 rep2 prot (fmol mgDW-1)</t>
+          <t>acetate(mmol/gDW)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>pryuvate(mmol/gDW)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>glycerol(mmol/gDW)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>galactose(mmol/gDW)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>raffinose(mmol/gDW)</t>
         </is>
       </c>
     </row>
@@ -477,28 +497,40 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3373</v>
+        <v>3638</v>
       </c>
       <c r="C2" t="n">
-        <v>3373</v>
+        <v>5003</v>
       </c>
       <c r="D2" t="n">
-        <v>3373</v>
+        <v>5003</v>
       </c>
       <c r="E2" t="n">
-        <v>3373</v>
+        <v>5003</v>
       </c>
       <c r="F2" t="n">
-        <v>3373</v>
+        <v>5003</v>
       </c>
       <c r="G2" t="n">
-        <v>3373</v>
+        <v>5003</v>
       </c>
       <c r="H2" t="n">
-        <v>3373</v>
+        <v>5003</v>
       </c>
       <c r="I2" t="n">
-        <v>3373</v>
+        <v>5003</v>
+      </c>
+      <c r="J2" t="n">
+        <v>5003</v>
+      </c>
+      <c r="K2" t="n">
+        <v>5003</v>
+      </c>
+      <c r="L2" t="n">
+        <v>4675</v>
+      </c>
+      <c r="M2" t="n">
+        <v>4675</v>
       </c>
     </row>
     <row r="3">
@@ -508,28 +540,40 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>14826.10135158759</v>
+        <v>25197.11143939522</v>
       </c>
       <c r="C3" t="n">
-        <v>15022.05319511131</v>
+        <v>18485.57923041054</v>
       </c>
       <c r="D3" t="n">
-        <v>8198.85862757145</v>
+        <v>19877.93171144229</v>
       </c>
       <c r="E3" t="n">
-        <v>8627.277122959313</v>
+        <v>19409.0015085981</v>
       </c>
       <c r="F3" t="n">
-        <v>11599.68999075906</v>
+        <v>19159.77728026655</v>
       </c>
       <c r="G3" t="n">
-        <v>11948.22655096345</v>
+        <v>18144.73355819078</v>
       </c>
       <c r="H3" t="n">
-        <v>6941.180029943468</v>
+        <v>18392.48050440425</v>
       </c>
       <c r="I3" t="n">
-        <v>7236.226913314021</v>
+        <v>22733.94674382204</v>
+      </c>
+      <c r="J3" t="n">
+        <v>20825.14545103406</v>
+      </c>
+      <c r="K3" t="n">
+        <v>19039.89691510175</v>
+      </c>
+      <c r="L3" t="n">
+        <v>17120.25161811963</v>
+      </c>
+      <c r="M3" t="n">
+        <v>16960.23272008139</v>
       </c>
     </row>
     <row r="4">
@@ -539,28 +583,40 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>94239.38851651702</v>
+        <v>150261.3272235484</v>
       </c>
       <c r="C4" t="n">
-        <v>85695.71635475392</v>
+        <v>111315.8457873329</v>
       </c>
       <c r="D4" t="n">
-        <v>42454.42587793225</v>
+        <v>121062.908847915</v>
       </c>
       <c r="E4" t="n">
-        <v>44033.23347275851</v>
+        <v>140739.2913885579</v>
       </c>
       <c r="F4" t="n">
-        <v>62084.95306620732</v>
+        <v>140222.1323186173</v>
       </c>
       <c r="G4" t="n">
-        <v>60256.58914780393</v>
+        <v>106428.738777524</v>
       </c>
       <c r="H4" t="n">
-        <v>35401.95458442126</v>
+        <v>106815.8881086667</v>
       </c>
       <c r="I4" t="n">
-        <v>38519.1452450217</v>
+        <v>145397.2715350767</v>
+      </c>
+      <c r="J4" t="n">
+        <v>140203.8699283449</v>
+      </c>
+      <c r="K4" t="n">
+        <v>112739.2075482871</v>
+      </c>
+      <c r="L4" t="n">
+        <v>136151.7548107124</v>
+      </c>
+      <c r="M4" t="n">
+        <v>122816.8832387086</v>
       </c>
     </row>
     <row r="5">
@@ -570,28 +626,40 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.06078645638446672</v>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>0.06286019476858504</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>0.03292059684787744</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>0.1929209646413877</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>0.04678872229166838</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>0.6524906584822536</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>0.1554674440333529</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>0.3918194431011597</v>
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -601,28 +669,40 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>202.8226243589605</v>
+        <v>218.3634347026226</v>
       </c>
       <c r="C6" t="n">
-        <v>218.7340473298869</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
-        <v>111.2426965584351</v>
+        <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>139.1037763717975</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>183.5705825883726</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>189.3802506806709</v>
+        <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>111.0704279515588</v>
+        <v>0</v>
       </c>
       <c r="I6" t="n">
-        <v>110.9447578581742</v>
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -632,28 +712,40 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>811.5168785687972</v>
+        <v>1156.420868978249</v>
       </c>
       <c r="C7" t="n">
-        <v>865.6256519359144</v>
+        <v>324.6317986632183</v>
       </c>
       <c r="D7" t="n">
-        <v>427.3430172600542</v>
+        <v>350.1456340418788</v>
       </c>
       <c r="E7" t="n">
-        <v>538.739589211688</v>
+        <v>370.9677987451415</v>
       </c>
       <c r="F7" t="n">
-        <v>678.1739868452653</v>
+        <v>377.6731503940441</v>
       </c>
       <c r="G7" t="n">
-        <v>724.7118121437436</v>
+        <v>353.6707032642191</v>
       </c>
       <c r="H7" t="n">
-        <v>424.7873287240129</v>
+        <v>364.8590157232369</v>
       </c>
       <c r="I7" t="n">
-        <v>435.1144108794591</v>
+        <v>339.2015691032469</v>
+      </c>
+      <c r="J7" t="n">
+        <v>392.5928287176063</v>
+      </c>
+      <c r="K7" t="n">
+        <v>387.7875861359022</v>
+      </c>
+      <c r="L7" t="n">
+        <v>532.1152826546157</v>
+      </c>
+      <c r="M7" t="n">
+        <v>486.2243460482219</v>
       </c>
     </row>
     <row r="8">
@@ -663,28 +755,40 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3494.894610431665</v>
+        <v>5416.39947840087</v>
       </c>
       <c r="C8" t="n">
-        <v>3854.610975794258</v>
+        <v>2714.763019572504</v>
       </c>
       <c r="D8" t="n">
-        <v>1898.764095805589</v>
+        <v>2936.210470480949</v>
       </c>
       <c r="E8" t="n">
-        <v>2350.879291307855</v>
+        <v>2999.314310180298</v>
       </c>
       <c r="F8" t="n">
-        <v>2979.463907653272</v>
+        <v>3111.551629923011</v>
       </c>
       <c r="G8" t="n">
-        <v>3131.00720347323</v>
+        <v>3002.571606630671</v>
       </c>
       <c r="H8" t="n">
-        <v>1827.41800098425</v>
+        <v>3003.576668248743</v>
       </c>
       <c r="I8" t="n">
-        <v>1911.728678718476</v>
+        <v>2876.622574639217</v>
+      </c>
+      <c r="J8" t="n">
+        <v>3230.32160578173</v>
+      </c>
+      <c r="K8" t="n">
+        <v>3245.43340987828</v>
+      </c>
+      <c r="L8" t="n">
+        <v>3418.42180444752</v>
+      </c>
+      <c r="M8" t="n">
+        <v>3241.058766830559</v>
       </c>
     </row>
     <row r="9">
@@ -694,28 +798,40 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3532728.342374335</v>
+        <v>2827568.866170935</v>
       </c>
       <c r="C9" t="n">
-        <v>2873851.595377475</v>
+        <v>3441293.778590984</v>
       </c>
       <c r="D9" t="n">
-        <v>942560.9738540711</v>
+        <v>2997519.452074238</v>
       </c>
       <c r="E9" t="n">
-        <v>990764.0790722463</v>
+        <v>3474572.365462308</v>
       </c>
       <c r="F9" t="n">
-        <v>1481068.682882923</v>
+        <v>3766905.59001234</v>
       </c>
       <c r="G9" t="n">
-        <v>1285386.303692142</v>
+        <v>2753403.630072502</v>
       </c>
       <c r="H9" t="n">
-        <v>674599.3665497858</v>
+        <v>2173211.290130805</v>
       </c>
       <c r="I9" t="n">
-        <v>1062372.807385358</v>
+        <v>3039979.376189653</v>
+      </c>
+      <c r="J9" t="n">
+        <v>6004868.809911354</v>
+      </c>
+      <c r="K9" t="n">
+        <v>2247437.265527637</v>
+      </c>
+      <c r="L9" t="n">
+        <v>5375654.536827597</v>
+      </c>
+      <c r="M9" t="n">
+        <v>4239740.357313359</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: rerun all the script
</commit_message>
<xml_diff>
--- a/data/proteomics/protein_copy_statistical.xlsx
+++ b/data/proteomics/protein_copy_statistical.xlsx
@@ -456,207 +456,207 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>prot.10</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>prot.11</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>prot.12</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>prot.13</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>prot.14</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>prot.15</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>prot.16</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>prot.17</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>prot.18</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>prot.19</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
           <t>prot.2</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>prot.20</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>prot.21</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>prot.22</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>prot.23</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>prot.24</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>prot.25</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>prot.26</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>prot.27</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>prot.28</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>prot.29</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>prot.3</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>prot.30</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>prot.31</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>prot.32</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>prot.33</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>prot.34</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>prot.35</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>prot.36</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>prot.37</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>prot.38</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>prot.39</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>prot.4</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>prot.40</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>prot.41</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>prot.42</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>prot.5</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>prot.6</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>prot.7</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>prot.8</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>prot.9</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>prot.10</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>prot.11</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>prot.12</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>prot.13</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>prot.14</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>prot.15</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>prot.16</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>prot.17</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>prot.18</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>prot.19</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>prot.20</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>prot.21</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>prot.22</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>prot.23</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>prot.24</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>prot.25</t>
-        </is>
-      </c>
-      <c r="AE1" s="1" t="inlineStr">
-        <is>
-          <t>prot.26</t>
-        </is>
-      </c>
-      <c r="AF1" s="1" t="inlineStr">
-        <is>
-          <t>prot.27</t>
-        </is>
-      </c>
-      <c r="AG1" s="1" t="inlineStr">
-        <is>
-          <t>prot.28</t>
-        </is>
-      </c>
-      <c r="AH1" s="1" t="inlineStr">
-        <is>
-          <t>prot.29</t>
-        </is>
-      </c>
-      <c r="AI1" s="1" t="inlineStr">
-        <is>
-          <t>prot.30</t>
-        </is>
-      </c>
-      <c r="AJ1" s="1" t="inlineStr">
-        <is>
-          <t>prot.31</t>
-        </is>
-      </c>
-      <c r="AK1" s="1" t="inlineStr">
-        <is>
-          <t>prot.32</t>
-        </is>
-      </c>
-      <c r="AL1" s="1" t="inlineStr">
-        <is>
-          <t>prot.33</t>
-        </is>
-      </c>
-      <c r="AM1" s="1" t="inlineStr">
-        <is>
-          <t>prot.34</t>
-        </is>
-      </c>
-      <c r="AN1" s="1" t="inlineStr">
-        <is>
-          <t>prot.35</t>
-        </is>
-      </c>
-      <c r="AO1" s="1" t="inlineStr">
-        <is>
-          <t>prot.36</t>
-        </is>
-      </c>
-      <c r="AP1" s="1" t="inlineStr">
-        <is>
-          <t>prot.37</t>
-        </is>
-      </c>
-      <c r="AQ1" s="1" t="inlineStr">
-        <is>
-          <t>prot.38</t>
-        </is>
-      </c>
-      <c r="AR1" s="1" t="inlineStr">
-        <is>
-          <t>prot.39</t>
-        </is>
-      </c>
-      <c r="AS1" s="1" t="inlineStr">
-        <is>
-          <t>prot.40</t>
-        </is>
-      </c>
-      <c r="AT1" s="1" t="inlineStr">
-        <is>
-          <t>prot.41</t>
-        </is>
-      </c>
-      <c r="AU1" s="1" t="inlineStr">
-        <is>
-          <t>prot.42</t>
         </is>
       </c>
       <c r="AV1" s="1" t="inlineStr">
@@ -829,130 +829,130 @@
         <v>3928</v>
       </c>
       <c r="F2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="G2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="H2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="I2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="J2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="K2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="L2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="M2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="N2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="O2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="P2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="Q2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="R2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="S2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="T2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="U2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="V2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="W2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="X2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="Y2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="Z2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="AA2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="AB2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="AC2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="AD2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="AE2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="AF2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="AG2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="AH2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="AI2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="AJ2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="AK2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="AL2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="AM2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="AN2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="AO2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="AP2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="AQ2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="AR2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="AS2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="AT2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="AU2" t="n">
-        <v>3127</v>
+        <v>3128</v>
       </c>
       <c r="AV2" t="n">
         <v>2142</v>
@@ -1018,31 +1018,31 @@
         <v>5391</v>
       </c>
       <c r="BQ2" t="n">
-        <v>2556</v>
+        <v>2561</v>
       </c>
       <c r="BR2" t="n">
-        <v>2520</v>
+        <v>2525</v>
       </c>
       <c r="BS2" t="n">
-        <v>2507</v>
+        <v>2512</v>
       </c>
       <c r="BT2" t="n">
-        <v>2464</v>
+        <v>2469</v>
       </c>
       <c r="BU2" t="n">
-        <v>2485</v>
+        <v>2490</v>
       </c>
       <c r="BV2" t="n">
-        <v>2468</v>
+        <v>2473</v>
       </c>
       <c r="BW2" t="n">
-        <v>2521</v>
+        <v>2526</v>
       </c>
       <c r="BX2" t="n">
-        <v>2433</v>
+        <v>2438</v>
       </c>
       <c r="BY2" t="n">
-        <v>2416</v>
+        <v>2421</v>
       </c>
     </row>
     <row r="3">
@@ -1052,7 +1052,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>31699.93008138768</v>
+        <v>31699.93008138769</v>
       </c>
       <c r="C3" t="n">
         <v>28687.47638216143</v>
@@ -1061,139 +1061,139 @@
         <v>25039.36838391844</v>
       </c>
       <c r="E3" t="n">
-        <v>27809.26232010379</v>
+        <v>27809.26232010378</v>
       </c>
       <c r="F3" t="n">
-        <v>12522.43267810243</v>
+        <v>12518.42934284728</v>
       </c>
       <c r="G3" t="n">
-        <v>11277.01671015698</v>
+        <v>14073.40599052339</v>
       </c>
       <c r="H3" t="n">
-        <v>12071.75420804332</v>
+        <v>12038.61901122389</v>
       </c>
       <c r="I3" t="n">
-        <v>17888.77354574347</v>
+        <v>12049.98975133031</v>
       </c>
       <c r="J3" t="n">
-        <v>19085.6475887543</v>
+        <v>13278.63061451924</v>
       </c>
       <c r="K3" t="n">
-        <v>16079.89758785596</v>
+        <v>12955.02173001969</v>
       </c>
       <c r="L3" t="n">
-        <v>9307.236004476186</v>
+        <v>13073.89329933087</v>
       </c>
       <c r="M3" t="n">
-        <v>9831.12797740136</v>
+        <v>22101.55608720983</v>
       </c>
       <c r="N3" t="n">
-        <v>12955.38369074964</v>
+        <v>22145.20565946272</v>
       </c>
       <c r="O3" t="n">
-        <v>14077.90660005026</v>
+        <v>20929.35619261183</v>
       </c>
       <c r="P3" t="n">
-        <v>12042.46890537523</v>
+        <v>27481.03484670626</v>
       </c>
       <c r="Q3" t="n">
-        <v>12053.84328179124</v>
+        <v>11273.41152578673</v>
       </c>
       <c r="R3" t="n">
-        <v>13282.87705859168</v>
+        <v>29003.88583055399</v>
       </c>
       <c r="S3" t="n">
-        <v>12959.1646854818</v>
+        <v>28923.62587780414</v>
       </c>
       <c r="T3" t="n">
-        <v>13078.07426936584</v>
+        <v>24828.64835487205</v>
       </c>
       <c r="U3" t="n">
-        <v>22108.6240616541</v>
+        <v>30025.26094565109</v>
       </c>
       <c r="V3" t="n">
-        <v>22152.28759283639</v>
+        <v>30818.38815773577</v>
       </c>
       <c r="W3" t="n">
-        <v>20936.04930300283</v>
+        <v>23716.62980526402</v>
       </c>
       <c r="X3" t="n">
-        <v>27489.82315334096</v>
+        <v>13994.52970436225</v>
       </c>
       <c r="Y3" t="n">
-        <v>29013.16113782311</v>
+        <v>17422.97033576227</v>
       </c>
       <c r="Z3" t="n">
-        <v>28932.87551831511</v>
+        <v>10019.73321055387</v>
       </c>
       <c r="AA3" t="n">
-        <v>24836.58844069068</v>
+        <v>16401.9036189057</v>
       </c>
       <c r="AB3" t="n">
-        <v>30034.86288391321</v>
+        <v>12067.89495158295</v>
       </c>
       <c r="AC3" t="n">
-        <v>30828.24373437719</v>
+        <v>16291.49478922326</v>
       </c>
       <c r="AD3" t="n">
-        <v>23724.21427274253</v>
+        <v>18880.99950768716</v>
       </c>
       <c r="AE3" t="n">
-        <v>13999.00508962109</v>
+        <v>23471.27299244677</v>
       </c>
       <c r="AF3" t="n">
-        <v>17428.54212032759</v>
+        <v>20160.17033812535</v>
       </c>
       <c r="AG3" t="n">
-        <v>10022.93747445235</v>
+        <v>18998.38899176757</v>
       </c>
       <c r="AH3" t="n">
-        <v>16407.14887110234</v>
+        <v>17108.93412808232</v>
       </c>
       <c r="AI3" t="n">
-        <v>16296.70473319167</v>
+        <v>18038.95622030722</v>
       </c>
       <c r="AJ3" t="n">
-        <v>18887.03756317411</v>
+        <v>14969.74580855612</v>
       </c>
       <c r="AK3" t="n">
-        <v>23478.77899596211</v>
+        <v>19545.68585555418</v>
       </c>
       <c r="AL3" t="n">
-        <v>20166.6174664714</v>
+        <v>16673.01648769615</v>
       </c>
       <c r="AM3" t="n">
-        <v>19004.46458786343</v>
+        <v>17883.05462836951</v>
       </c>
       <c r="AN3" t="n">
-        <v>17114.40548533466</v>
+        <v>22750.91520827561</v>
       </c>
       <c r="AO3" t="n">
-        <v>18044.72499428237</v>
+        <v>21842.0061224755</v>
       </c>
       <c r="AP3" t="n">
-        <v>14974.53306337178</v>
+        <v>21217.03775782351</v>
       </c>
       <c r="AQ3" t="n">
-        <v>19551.93647463176</v>
+        <v>19079.54603901364</v>
       </c>
       <c r="AR3" t="n">
-        <v>16678.34844052241</v>
+        <v>16074.75695563478</v>
       </c>
       <c r="AS3" t="n">
-        <v>22758.19084473492</v>
+        <v>9304.260545395471</v>
       </c>
       <c r="AT3" t="n">
-        <v>21848.99109405288</v>
+        <v>9827.985033674569</v>
       </c>
       <c r="AU3" t="n">
-        <v>21223.82286743586</v>
+        <v>12951.24194404544</v>
       </c>
       <c r="AV3" t="n">
         <v>26692.50099691877</v>
       </c>
       <c r="AW3" t="n">
-        <v>30739.82382791223</v>
+        <v>30739.82382791224</v>
       </c>
       <c r="AX3" t="n">
         <v>31699.64696088852</v>
@@ -1250,34 +1250,34 @@
         <v>11388.10700346718</v>
       </c>
       <c r="BP3" t="n">
-        <v>7764.094734708287</v>
+        <v>7764.094734708288</v>
       </c>
       <c r="BQ3" t="n">
-        <v>29068.32665296084</v>
+        <v>29011.57474618037</v>
       </c>
       <c r="BR3" t="n">
-        <v>30322.7002055345</v>
+        <v>30262.65525463245</v>
       </c>
       <c r="BS3" t="n">
-        <v>33520.00698071731</v>
+        <v>33453.28722159965</v>
       </c>
       <c r="BT3" t="n">
-        <v>37364.5365335106</v>
+        <v>37288.8691853261</v>
       </c>
       <c r="BU3" t="n">
-        <v>27443.26053025264</v>
+        <v>27388.1535813967</v>
       </c>
       <c r="BV3" t="n">
-        <v>31954.37323410008</v>
+        <v>31889.76673746826</v>
       </c>
       <c r="BW3" t="n">
-        <v>32217.23285142431</v>
+        <v>32153.46160666694</v>
       </c>
       <c r="BX3" t="n">
-        <v>34551.55819569284</v>
+        <v>34480.69774000028</v>
       </c>
       <c r="BY3" t="n">
-        <v>31349.45089406132</v>
+        <v>31284.70605537057</v>
       </c>
     </row>
     <row r="4">
@@ -1299,133 +1299,133 @@
         <v>141223.2894959995</v>
       </c>
       <c r="F4" t="n">
-        <v>66936.03740698223</v>
+        <v>66918.75512960671</v>
       </c>
       <c r="G4" t="n">
-        <v>60532.97477119041</v>
+        <v>71709.43327629076</v>
       </c>
       <c r="H4" t="n">
-        <v>67838.1793838442</v>
+        <v>63891.0400374174</v>
       </c>
       <c r="I4" t="n">
-        <v>113019.7647040295</v>
+        <v>62268.56123348384</v>
       </c>
       <c r="J4" t="n">
-        <v>123933.3220014994</v>
+        <v>65786.07688594142</v>
       </c>
       <c r="K4" t="n">
-        <v>96388.77551727369</v>
+        <v>64565.5174438578</v>
       </c>
       <c r="L4" t="n">
-        <v>51497.44346481315</v>
+        <v>68284.49105461262</v>
       </c>
       <c r="M4" t="n">
-        <v>53751.59961656742</v>
+        <v>116896.4757637392</v>
       </c>
       <c r="N4" t="n">
-        <v>68179.03059273884</v>
+        <v>114124.7746417368</v>
       </c>
       <c r="O4" t="n">
-        <v>71730.57130375157</v>
+        <v>106860.0609547023</v>
       </c>
       <c r="P4" t="n">
-        <v>63910.56945756701</v>
+        <v>142647.5166379431</v>
       </c>
       <c r="Q4" t="n">
-        <v>62287.14171905869</v>
+        <v>60518.16560546382</v>
       </c>
       <c r="R4" t="n">
-        <v>65805.45903293697</v>
+        <v>153554.5969986021</v>
       </c>
       <c r="S4" t="n">
-        <v>64587.44229582025</v>
+        <v>149557.2542187138</v>
       </c>
       <c r="T4" t="n">
-        <v>68304.71623225568</v>
+        <v>175499.2435029291</v>
       </c>
       <c r="U4" t="n">
-        <v>116929.0576506173</v>
+        <v>207095.757270361</v>
       </c>
       <c r="V4" t="n">
-        <v>114159.22677532</v>
+        <v>207590.2535045513</v>
       </c>
       <c r="W4" t="n">
-        <v>106894.8860790297</v>
+        <v>134082.8838197027</v>
       </c>
       <c r="X4" t="n">
-        <v>142692.8716278319</v>
+        <v>75151.72501234972</v>
       </c>
       <c r="Y4" t="n">
-        <v>153601.502919268</v>
+        <v>96112.14596625253</v>
       </c>
       <c r="Z4" t="n">
-        <v>149600.8276335788</v>
+        <v>49828.48776493017</v>
       </c>
       <c r="AA4" t="n">
-        <v>175532.0703759744</v>
+        <v>81158.16824771844</v>
       </c>
       <c r="AB4" t="n">
-        <v>207135.2867813307</v>
+        <v>67819.35466305827</v>
       </c>
       <c r="AC4" t="n">
-        <v>207630.4125781679</v>
+        <v>80526.3478628739</v>
       </c>
       <c r="AD4" t="n">
-        <v>134114.4493142845</v>
+        <v>103059.9498914771</v>
       </c>
       <c r="AE4" t="n">
-        <v>75171.09024679731</v>
+        <v>135538.6127013691</v>
       </c>
       <c r="AF4" t="n">
-        <v>96135.85665352779</v>
+        <v>109537.1553925181</v>
       </c>
       <c r="AG4" t="n">
-        <v>49843.38100575726</v>
+        <v>100658.6485246631</v>
       </c>
       <c r="AH4" t="n">
-        <v>81180.39803944319</v>
+        <v>86439.74708679192</v>
       </c>
       <c r="AI4" t="n">
-        <v>80549.71077916134</v>
+        <v>89448.19028639616</v>
       </c>
       <c r="AJ4" t="n">
-        <v>103085.5230209689</v>
+        <v>82218.62331929988</v>
       </c>
       <c r="AK4" t="n">
-        <v>135571.0612910033</v>
+        <v>113109.3165817835</v>
       </c>
       <c r="AL4" t="n">
-        <v>109564.778723442</v>
+        <v>90413.41583845747</v>
       </c>
       <c r="AM4" t="n">
-        <v>100684.6235071302</v>
+        <v>112992.8999783003</v>
       </c>
       <c r="AN4" t="n">
-        <v>86462.43162682682</v>
+        <v>118705.3108374197</v>
       </c>
       <c r="AO4" t="n">
-        <v>89473.92721309305</v>
+        <v>116894.1264883224</v>
       </c>
       <c r="AP4" t="n">
-        <v>82237.74954078115</v>
+        <v>113008.3704132263</v>
       </c>
       <c r="AQ4" t="n">
-        <v>113134.1287620463</v>
+        <v>123906.1068952232</v>
       </c>
       <c r="AR4" t="n">
-        <v>90434.90184809137</v>
+        <v>96366.74830504799</v>
       </c>
       <c r="AS4" t="n">
-        <v>118737.5902741415</v>
+        <v>51483.08474887283</v>
       </c>
       <c r="AT4" t="n">
-        <v>116920.723352011</v>
+        <v>53737.12567912344</v>
       </c>
       <c r="AU4" t="n">
-        <v>113037.0564166722</v>
+        <v>68154.49267078238</v>
       </c>
       <c r="AV4" t="n">
-        <v>84421.98038418526</v>
+        <v>84421.98038418527</v>
       </c>
       <c r="AW4" t="n">
         <v>175075.6849168531</v>
@@ -1488,31 +1488,31 @@
         <v>27505.07111669971</v>
       </c>
       <c r="BQ4" t="n">
-        <v>120732.9908766626</v>
+        <v>119518.5718200878</v>
       </c>
       <c r="BR4" t="n">
-        <v>116672.5530703134</v>
+        <v>115424.9224959265</v>
       </c>
       <c r="BS4" t="n">
-        <v>101701.5896552759</v>
+        <v>99572.66923928485</v>
       </c>
       <c r="BT4" t="n">
-        <v>103453.4782046555</v>
+        <v>100702.5203317217</v>
       </c>
       <c r="BU4" t="n">
-        <v>73029.99571240647</v>
+        <v>70673.84324781052</v>
       </c>
       <c r="BV4" t="n">
-        <v>85832.6813934923</v>
+        <v>82860.57921750014</v>
       </c>
       <c r="BW4" t="n">
-        <v>86498.88595830589</v>
+        <v>83422.5148094544</v>
       </c>
       <c r="BX4" t="n">
-        <v>92359.27389715347</v>
+        <v>89262.80278051979</v>
       </c>
       <c r="BY4" t="n">
-        <v>84989.72081612758</v>
+        <v>82206.88924311596</v>
       </c>
     </row>
     <row r="5">
@@ -1769,130 +1769,130 @@
         <v>598.8225460547256</v>
       </c>
       <c r="F6" t="n">
-        <v>80.10982895236199</v>
+        <v>80.153840101566</v>
       </c>
       <c r="G6" t="n">
-        <v>71.9021966408427</v>
+        <v>89.22383774915599</v>
       </c>
       <c r="H6" t="n">
-        <v>72.23298898596441</v>
+        <v>75.04330767897702</v>
       </c>
       <c r="I6" t="n">
-        <v>101.271074096038</v>
+        <v>78.29737540315185</v>
       </c>
       <c r="J6" t="n">
-        <v>102.118304691007</v>
+        <v>87.24983850770549</v>
       </c>
       <c r="K6" t="n">
-        <v>88.87006471788501</v>
+        <v>84.6444452708525</v>
       </c>
       <c r="L6" t="n">
-        <v>60.92282654908671</v>
+        <v>86.74419417349949</v>
       </c>
       <c r="M6" t="n">
-        <v>64.3424964322008</v>
+        <v>116.063392636037</v>
       </c>
       <c r="N6" t="n">
-        <v>68.3089368501914</v>
+        <v>122.228649425091</v>
       </c>
       <c r="O6" t="n">
-        <v>89.035311589862</v>
+        <v>113.495998162415</v>
       </c>
       <c r="P6" t="n">
-        <v>75.040141621049</v>
+        <v>126.504210566316</v>
       </c>
       <c r="Q6" t="n">
-        <v>78.2617945859057</v>
+        <v>71.92754186199616</v>
       </c>
       <c r="R6" t="n">
-        <v>87.20702835194899</v>
+        <v>124.7542174007305</v>
       </c>
       <c r="S6" t="n">
-        <v>84.542629938041</v>
+        <v>132.988979687377</v>
       </c>
       <c r="T6" t="n">
-        <v>86.737089080213</v>
+        <v>129.9786733350215</v>
       </c>
       <c r="U6" t="n">
-        <v>116.000188102348</v>
+        <v>149.069780098371</v>
       </c>
       <c r="V6" t="n">
-        <v>122.161784694796</v>
+        <v>150.3660340050165</v>
       </c>
       <c r="W6" t="n">
-        <v>113.450765838454</v>
+        <v>131.6739927493375</v>
       </c>
       <c r="X6" t="n">
-        <v>126.452653760554</v>
+        <v>79.3925757582485</v>
       </c>
       <c r="Y6" t="n">
-        <v>124.560238196801</v>
+        <v>97.94365716367651</v>
       </c>
       <c r="Z6" t="n">
-        <v>132.877199231084</v>
+        <v>57.02712346285405</v>
       </c>
       <c r="AA6" t="n">
-        <v>129.963492116227</v>
+        <v>97.682689048824</v>
       </c>
       <c r="AB6" t="n">
-        <v>149.03755972754</v>
+        <v>72.25688582135211</v>
       </c>
       <c r="AC6" t="n">
-        <v>150.268812572461</v>
+        <v>101.874785070135</v>
       </c>
       <c r="AD6" t="n">
-        <v>131.654940164231</v>
+        <v>115.6961743309295</v>
       </c>
       <c r="AE6" t="n">
-        <v>79.337552171515</v>
+        <v>132.0487719595385</v>
       </c>
       <c r="AF6" t="n">
-        <v>97.911141746407</v>
+        <v>116.195795571911</v>
       </c>
       <c r="AG6" t="n">
-        <v>56.9763669037585</v>
+        <v>127.8639982888895</v>
       </c>
       <c r="AH6" t="n">
-        <v>97.67975451808201</v>
+        <v>109.2292227418975</v>
       </c>
       <c r="AI6" t="n">
-        <v>101.851790787538</v>
+        <v>113.1034768798825</v>
       </c>
       <c r="AJ6" t="n">
-        <v>115.652917250189</v>
+        <v>93.56920149865749</v>
       </c>
       <c r="AK6" t="n">
-        <v>132.020056970593</v>
+        <v>118.2239190105435</v>
       </c>
       <c r="AL6" t="n">
-        <v>116.115144208074</v>
+        <v>92.42240277526301</v>
       </c>
       <c r="AM6" t="n">
-        <v>127.737541283561</v>
+        <v>101.349335335127</v>
       </c>
       <c r="AN6" t="n">
-        <v>109.164391900025</v>
+        <v>115.4205619258175</v>
       </c>
       <c r="AO6" t="n">
-        <v>112.952652871421</v>
+        <v>123.6904722433875</v>
       </c>
       <c r="AP6" t="n">
-        <v>93.375223351751</v>
+        <v>114.9420963933715</v>
       </c>
       <c r="AQ6" t="n">
-        <v>118.115934460865</v>
+        <v>102.1709409717205</v>
       </c>
       <c r="AR6" t="n">
-        <v>92.399422273114</v>
+        <v>88.87837446505051</v>
       </c>
       <c r="AS6" t="n">
-        <v>115.280845310785</v>
+        <v>60.94255695019196</v>
       </c>
       <c r="AT6" t="n">
-        <v>123.625635998953</v>
+        <v>64.34762314643191</v>
       </c>
       <c r="AU6" t="n">
-        <v>114.800815775789</v>
+        <v>68.32148353311601</v>
       </c>
       <c r="AV6" t="n">
         <v>276.1309466666666</v>
@@ -1958,31 +1958,31 @@
         <v>1391.58692875209</v>
       </c>
       <c r="BQ6" t="n">
-        <v>1256.57572389893</v>
+        <v>1260.80884481044</v>
       </c>
       <c r="BR6" t="n">
-        <v>1379.640008760082</v>
+        <v>1381.107826577527</v>
       </c>
       <c r="BS6" t="n">
-        <v>1670.31167326096</v>
+        <v>1673.709179843117</v>
       </c>
       <c r="BT6" t="n">
-        <v>1896.166258715754</v>
+        <v>1898.452614922407</v>
       </c>
       <c r="BU6" t="n">
-        <v>1386.588015489567</v>
+        <v>1391.751271143925</v>
       </c>
       <c r="BV6" t="n">
-        <v>1552.23531400505</v>
+        <v>1555.49256997255</v>
       </c>
       <c r="BW6" t="n">
-        <v>1468.786393033914</v>
+        <v>1470.140640415737</v>
       </c>
       <c r="BX6" t="n">
-        <v>1615.812485984597</v>
+        <v>1618.886195773877</v>
       </c>
       <c r="BY6" t="n">
-        <v>1438.217894773078</v>
+        <v>1438.82437619788</v>
       </c>
     </row>
     <row r="7">
@@ -2004,130 +2004,130 @@
         <v>1620.066104975529</v>
       </c>
       <c r="F7" t="n">
-        <v>409.1146523443101</v>
+        <v>409.4435183511421</v>
       </c>
       <c r="G7" t="n">
-        <v>376.4483348628201</v>
+        <v>478.665042327032</v>
       </c>
       <c r="H7" t="n">
-        <v>376.7999162156241</v>
+        <v>411.748567076176</v>
       </c>
       <c r="I7" t="n">
-        <v>514.5590160258899</v>
+        <v>424.8076508259981</v>
       </c>
       <c r="J7" t="n">
-        <v>531.182851432904</v>
+        <v>470.727020671435</v>
       </c>
       <c r="K7" t="n">
-        <v>475.195991496512</v>
+        <v>450.7232738490241</v>
       </c>
       <c r="L7" t="n">
-        <v>324.131100020992</v>
+        <v>474.0527023047971</v>
       </c>
       <c r="M7" t="n">
-        <v>343.607094873152</v>
+        <v>626.452890847641</v>
       </c>
       <c r="N7" t="n">
-        <v>363.210100982608</v>
+        <v>630.4970199740851</v>
       </c>
       <c r="O7" t="n">
-        <v>478.060984375348</v>
+        <v>611.6755832087121</v>
       </c>
       <c r="P7" t="n">
-        <v>411.362582286854</v>
+        <v>684.2520752452881</v>
       </c>
       <c r="Q7" t="n">
-        <v>424.7358915702761</v>
+        <v>376.9176106373041</v>
       </c>
       <c r="R7" t="n">
-        <v>470.320363213514</v>
+        <v>689.6186369993579</v>
       </c>
       <c r="S7" t="n">
-        <v>450.499508656956</v>
+        <v>720.433652805405</v>
       </c>
       <c r="T7" t="n">
-        <v>474.0383334864761</v>
+        <v>664.8991028762611</v>
       </c>
       <c r="U7" t="n">
-        <v>625.5640711738</v>
+        <v>776.621375259928</v>
       </c>
       <c r="V7" t="n">
-        <v>629.568824157746</v>
+        <v>776.7648332078691</v>
       </c>
       <c r="W7" t="n">
-        <v>611.6392044702501</v>
+        <v>728.987666750442</v>
       </c>
       <c r="X7" t="n">
-        <v>683.8434919306101</v>
+        <v>446.007662366497</v>
       </c>
       <c r="Y7" t="n">
-        <v>689.4059805709339</v>
+        <v>544.379910508962</v>
       </c>
       <c r="Z7" t="n">
-        <v>719.903091581212</v>
+        <v>324.486787399214</v>
       </c>
       <c r="AA7" t="n">
-        <v>663.121538029126</v>
+        <v>567.3069295648041</v>
       </c>
       <c r="AB7" t="n">
-        <v>776.20511208592</v>
+        <v>379.044440547509</v>
       </c>
       <c r="AC7" t="n">
-        <v>776.1390838523081</v>
+        <v>569.4003721116369</v>
       </c>
       <c r="AD7" t="n">
-        <v>728.0230369564021</v>
+        <v>639.884285110873</v>
       </c>
       <c r="AE7" t="n">
-        <v>445.713054749138</v>
+        <v>728.6802569011461</v>
       </c>
       <c r="AF7" t="n">
-        <v>543.607995895514</v>
+        <v>656.760788633675</v>
       </c>
       <c r="AG7" t="n">
-        <v>324.215117924786</v>
+        <v>670.1065319708759</v>
       </c>
       <c r="AH7" t="n">
-        <v>565.7950062248221</v>
+        <v>612.772134210181</v>
       </c>
       <c r="AI7" t="n">
-        <v>568.7645827601319</v>
+        <v>636.982374490143</v>
       </c>
       <c r="AJ7" t="n">
-        <v>639.668711807906</v>
+        <v>476.126848074636</v>
       </c>
       <c r="AK7" t="n">
-        <v>727.000622220488</v>
+        <v>625.394497241151</v>
       </c>
       <c r="AL7" t="n">
-        <v>656.1467834300281</v>
+        <v>505.698484358969</v>
       </c>
       <c r="AM7" t="n">
-        <v>669.8259814675</v>
+        <v>514.6142165856779</v>
       </c>
       <c r="AN7" t="n">
-        <v>612.601290988654</v>
+        <v>671.6311782269211</v>
       </c>
       <c r="AO7" t="n">
-        <v>636.717357879328</v>
+        <v>699.7108922387761</v>
       </c>
       <c r="AP7" t="n">
-        <v>475.960701128</v>
+        <v>646.1137827467951</v>
       </c>
       <c r="AQ7" t="n">
-        <v>625.36432632047</v>
+        <v>533.4806050158311</v>
       </c>
       <c r="AR7" t="n">
-        <v>504.8455358959541</v>
+        <v>476.902489790331</v>
       </c>
       <c r="AS7" t="n">
-        <v>669.9725276060079</v>
+        <v>324.219424393084</v>
       </c>
       <c r="AT7" t="n">
-        <v>698.640819859202</v>
+        <v>343.837403115888</v>
       </c>
       <c r="AU7" t="n">
-        <v>646.0610133790561</v>
+        <v>363.4444094310151</v>
       </c>
       <c r="AV7" t="n">
         <v>3150.189533333333</v>
@@ -2193,31 +2193,31 @@
         <v>2621.81339062411</v>
       </c>
       <c r="BQ7" t="n">
-        <v>3878.485182046827</v>
+        <v>3897.2607425643</v>
       </c>
       <c r="BR7" t="n">
-        <v>4146.847632740117</v>
+        <v>4185.50432441001</v>
       </c>
       <c r="BS7" t="n">
-        <v>5222.147204366437</v>
+        <v>5257.817942003833</v>
       </c>
       <c r="BT7" t="n">
-        <v>6016.914090109292</v>
+        <v>6092.035543894624</v>
       </c>
       <c r="BU7" t="n">
-        <v>4393.528889509893</v>
+        <v>4413.418265632176</v>
       </c>
       <c r="BV7" t="n">
-        <v>4919.754784604967</v>
+        <v>4947.35745394813</v>
       </c>
       <c r="BW7" t="n">
-        <v>4680.707966273835</v>
+        <v>4699.517335925983</v>
       </c>
       <c r="BX7" t="n">
-        <v>4969.841710900063</v>
+        <v>4984.982889536515</v>
       </c>
       <c r="BY7" t="n">
-        <v>4556.437668683825</v>
+        <v>4602.083347639634</v>
       </c>
     </row>
     <row r="8">
@@ -2239,130 +2239,130 @@
         <v>5549.373053125927</v>
       </c>
       <c r="F8" t="n">
-        <v>2346.79385456043</v>
+        <v>2348.513731007125</v>
       </c>
       <c r="G8" t="n">
-        <v>2103.37546438965</v>
+        <v>2791.020711991105</v>
       </c>
       <c r="H8" t="n">
-        <v>2241.47875304705</v>
+        <v>2404.5715041502</v>
       </c>
       <c r="I8" t="n">
-        <v>3026.611200692641</v>
+        <v>2484.190718108605</v>
       </c>
       <c r="J8" t="n">
-        <v>3210.16161447828</v>
+        <v>2662.886714226255</v>
       </c>
       <c r="K8" t="n">
-        <v>2724.50331534326</v>
+        <v>2612.375236091995</v>
       </c>
       <c r="L8" t="n">
-        <v>1887.29544417095</v>
+        <v>2646.53807440495</v>
       </c>
       <c r="M8" t="n">
-        <v>1979.98545357657</v>
+        <v>3666.157091164975</v>
       </c>
       <c r="N8" t="n">
-        <v>2192.14407545276</v>
+        <v>3719.930911843795</v>
       </c>
       <c r="O8" t="n">
-        <v>2788.08140839877</v>
+        <v>3372.427067543215</v>
       </c>
       <c r="P8" t="n">
-        <v>2388.70219156998</v>
+        <v>3997.622913988991</v>
       </c>
       <c r="Q8" t="n">
-        <v>2481.76863152977</v>
+        <v>2107.94539919381</v>
       </c>
       <c r="R8" t="n">
-        <v>2661.57315468033</v>
+        <v>3991.597599254485</v>
       </c>
       <c r="S8" t="n">
-        <v>2610.95758013805</v>
+        <v>4212.478168900156</v>
       </c>
       <c r="T8" t="n">
-        <v>2642.16127845186</v>
+        <v>3768.6718179253</v>
       </c>
       <c r="U8" t="n">
-        <v>3657.39156096699</v>
+        <v>4445.64748534775</v>
       </c>
       <c r="V8" t="n">
-        <v>3703.60784336631</v>
+        <v>4522.843769262116</v>
       </c>
       <c r="W8" t="n">
-        <v>3367.56744051354</v>
+        <v>4113.171888843324</v>
       </c>
       <c r="X8" t="n">
-        <v>3994.27594618305</v>
+        <v>2498.566953207655</v>
       </c>
       <c r="Y8" t="n">
-        <v>3986.11098807064</v>
+        <v>3215.818705854976</v>
       </c>
       <c r="Z8" t="n">
-        <v>4210.270802058641</v>
+        <v>1916.923716843795</v>
       </c>
       <c r="AA8" t="n">
-        <v>3762.86629252787</v>
+        <v>3324.135993063216</v>
       </c>
       <c r="AB8" t="n">
-        <v>4442.41580586595</v>
+        <v>2253.25550433335</v>
       </c>
       <c r="AC8" t="n">
-        <v>4514.99869547551</v>
+        <v>3377.82491698234</v>
       </c>
       <c r="AD8" t="n">
-        <v>4094.10290833137</v>
+        <v>3667.645372110665</v>
       </c>
       <c r="AE8" t="n">
-        <v>2495.90525125942</v>
+        <v>4365.986547559615</v>
       </c>
       <c r="AF8" t="n">
-        <v>3213.46448837403</v>
+        <v>3730.977734331485</v>
       </c>
       <c r="AG8" t="n">
-        <v>1915.87728736745</v>
+        <v>3866.860856773311</v>
       </c>
       <c r="AH8" t="n">
-        <v>3323.139458204391</v>
+        <v>3571.558782545876</v>
       </c>
       <c r="AI8" t="n">
-        <v>3375.94534060718</v>
+        <v>3630.414992566505</v>
       </c>
       <c r="AJ8" t="n">
-        <v>3665.13758014954</v>
+        <v>2763.636521657936</v>
       </c>
       <c r="AK8" t="n">
-        <v>4357.682432565</v>
+        <v>3483.39701993602</v>
       </c>
       <c r="AL8" t="n">
-        <v>3726.315669206901</v>
+        <v>2973.50601361462</v>
       </c>
       <c r="AM8" t="n">
-        <v>3859.797579316691</v>
+        <v>3029.642681192711</v>
       </c>
       <c r="AN8" t="n">
-        <v>3565.22844190128</v>
+        <v>4051.887410421016</v>
       </c>
       <c r="AO8" t="n">
-        <v>3629.00075118834</v>
+        <v>4146.83148829323</v>
       </c>
       <c r="AP8" t="n">
-        <v>2758.228973445551</v>
+        <v>3832.676482595455</v>
       </c>
       <c r="AQ8" t="n">
-        <v>3474.5808186001</v>
+        <v>3212.952900399495</v>
       </c>
       <c r="AR8" t="n">
-        <v>2968.15305496358</v>
+        <v>2727.68302374458</v>
       </c>
       <c r="AS8" t="n">
-        <v>4043.595358407771</v>
+        <v>1888.27148433253</v>
       </c>
       <c r="AT8" t="n">
-        <v>4141.05254741574</v>
+        <v>1983.447830481315</v>
       </c>
       <c r="AU8" t="n">
-        <v>3826.54578971467</v>
+        <v>2201.31825328723</v>
       </c>
       <c r="AV8" t="n">
         <v>24083.15983333333</v>
@@ -2428,31 +2428,31 @@
         <v>5354.31353239906</v>
       </c>
       <c r="BQ8" t="n">
-        <v>17772.44853364126</v>
+        <v>17843.82832670887</v>
       </c>
       <c r="BR8" t="n">
-        <v>18106.01818306278</v>
+        <v>18154.2537715125</v>
       </c>
       <c r="BS8" t="n">
-        <v>21049.81994745378</v>
+        <v>21061.78915458805</v>
       </c>
       <c r="BT8" t="n">
-        <v>23773.5869697374</v>
+        <v>24091.71662989247</v>
       </c>
       <c r="BU8" t="n">
-        <v>17268.17173946237</v>
+        <v>17285.91237303745</v>
       </c>
       <c r="BV8" t="n">
-        <v>19295.91794866593</v>
+        <v>19387.33666661473</v>
       </c>
       <c r="BW8" t="n">
-        <v>18321.80229355223</v>
+        <v>18487.02942640524</v>
       </c>
       <c r="BX8" t="n">
-        <v>19259.2137137207</v>
+        <v>19323.62305194343</v>
       </c>
       <c r="BY8" t="n">
-        <v>17393.99753666686</v>
+        <v>17465.30152705693</v>
       </c>
     </row>
     <row r="9">
@@ -2477,127 +2477,127 @@
         <v>1698316.65470918</v>
       </c>
       <c r="G9" t="n">
+        <v>1953657.1430926</v>
+      </c>
+      <c r="H9" t="n">
+        <v>2014199.06168294</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1790822.73193406</v>
+      </c>
+      <c r="J9" t="n">
+        <v>1443755.52817518</v>
+      </c>
+      <c r="K9" t="n">
+        <v>1564591.58663698</v>
+      </c>
+      <c r="L9" t="n">
+        <v>1970313.74127984</v>
+      </c>
+      <c r="M9" t="n">
+        <v>2470661.90715718</v>
+      </c>
+      <c r="N9" t="n">
+        <v>2527283.75416462</v>
+      </c>
+      <c r="O9" t="n">
+        <v>2105847.42581576</v>
+      </c>
+      <c r="P9" t="n">
+        <v>2421202.90838998</v>
+      </c>
+      <c r="Q9" t="n">
         <v>1466816.39147648</v>
       </c>
-      <c r="H9" t="n">
+      <c r="R9" t="n">
+        <v>2861788.170666261</v>
+      </c>
+      <c r="S9" t="n">
+        <v>2785112.37681754</v>
+      </c>
+      <c r="T9" t="n">
+        <v>5038810.982452061</v>
+      </c>
+      <c r="U9" t="n">
+        <v>5636538.305159081</v>
+      </c>
+      <c r="V9" t="n">
+        <v>6049808.34863592</v>
+      </c>
+      <c r="W9" t="n">
+        <v>3456150.8082959</v>
+      </c>
+      <c r="X9" t="n">
+        <v>1599383.84789106</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>2408499.85809554</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>1153911.62847246</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>1847383.16277328</v>
+      </c>
+      <c r="AB9" t="n">
         <v>1924986.18972528</v>
       </c>
-      <c r="I9" t="n">
+      <c r="AC9" t="n">
+        <v>1963689.22389178</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>2583918.8280532</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>3856207.218654341</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>2799825.38531674</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>3081100.34485264</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>2326375.29938</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>1977546.07586316</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>2151719.3254238</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>3293436.0035962</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>1824004.88094594</v>
+      </c>
+      <c r="AM9" t="n">
         <v>2693794.69019408</v>
       </c>
-      <c r="J9" t="n">
+      <c r="AN9" t="n">
+        <v>2287799.90739608</v>
+      </c>
+      <c r="AO9" t="n">
+        <v>3008709.25558984</v>
+      </c>
+      <c r="AP9" t="n">
+        <v>2736623.22405714</v>
+      </c>
+      <c r="AQ9" t="n">
         <v>3265940.9522993</v>
       </c>
-      <c r="K9" t="n">
+      <c r="AR9" t="n">
         <v>2398317.22903388</v>
       </c>
-      <c r="L9" t="n">
+      <c r="AS9" t="n">
         <v>1673813.56260536</v>
       </c>
-      <c r="M9" t="n">
+      <c r="AT9" t="n">
         <v>1671361.1306579</v>
       </c>
-      <c r="N9" t="n">
+      <c r="AU9" t="n">
         <v>1447457.46153008</v>
-      </c>
-      <c r="O9" t="n">
-        <v>1953657.1430926</v>
-      </c>
-      <c r="P9" t="n">
-        <v>2014199.06168294</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>1790822.73193406</v>
-      </c>
-      <c r="R9" t="n">
-        <v>1443755.52817518</v>
-      </c>
-      <c r="S9" t="n">
-        <v>1564591.58663698</v>
-      </c>
-      <c r="T9" t="n">
-        <v>1970313.74127984</v>
-      </c>
-      <c r="U9" t="n">
-        <v>2470661.90715718</v>
-      </c>
-      <c r="V9" t="n">
-        <v>2527283.75416462</v>
-      </c>
-      <c r="W9" t="n">
-        <v>2105847.42581576</v>
-      </c>
-      <c r="X9" t="n">
-        <v>2421202.90838998</v>
-      </c>
-      <c r="Y9" t="n">
-        <v>2861788.170666261</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>2785112.37681754</v>
-      </c>
-      <c r="AA9" t="n">
-        <v>5038810.982452061</v>
-      </c>
-      <c r="AB9" t="n">
-        <v>5636538.305159081</v>
-      </c>
-      <c r="AC9" t="n">
-        <v>6049808.34863592</v>
-      </c>
-      <c r="AD9" t="n">
-        <v>3456150.8082959</v>
-      </c>
-      <c r="AE9" t="n">
-        <v>1599383.84789106</v>
-      </c>
-      <c r="AF9" t="n">
-        <v>2408499.85809554</v>
-      </c>
-      <c r="AG9" t="n">
-        <v>1153911.62847246</v>
-      </c>
-      <c r="AH9" t="n">
-        <v>1847383.16277328</v>
-      </c>
-      <c r="AI9" t="n">
-        <v>1963689.22389178</v>
-      </c>
-      <c r="AJ9" t="n">
-        <v>2583918.8280532</v>
-      </c>
-      <c r="AK9" t="n">
-        <v>3856207.218654341</v>
-      </c>
-      <c r="AL9" t="n">
-        <v>2799825.38531674</v>
-      </c>
-      <c r="AM9" t="n">
-        <v>3081100.34485264</v>
-      </c>
-      <c r="AN9" t="n">
-        <v>2326375.29938</v>
-      </c>
-      <c r="AO9" t="n">
-        <v>1977546.07586316</v>
-      </c>
-      <c r="AP9" t="n">
-        <v>2151719.3254238</v>
-      </c>
-      <c r="AQ9" t="n">
-        <v>3293436.0035962</v>
-      </c>
-      <c r="AR9" t="n">
-        <v>1824004.88094594</v>
-      </c>
-      <c r="AS9" t="n">
-        <v>2287799.90739608</v>
-      </c>
-      <c r="AT9" t="n">
-        <v>3008709.25558984</v>
-      </c>
-      <c r="AU9" t="n">
-        <v>2736623.22405714</v>
       </c>
       <c r="AV9" t="n">
         <v>2040565.936933333</v>
@@ -2672,22 +2672,22 @@
         <v>2186908.808510384</v>
       </c>
       <c r="BT9" t="n">
-        <v>1526611.414481163</v>
+        <v>1465364.870438074</v>
       </c>
       <c r="BU9" t="n">
-        <v>1197000.573967651</v>
+        <v>1073011.442711933</v>
       </c>
       <c r="BV9" t="n">
-        <v>1459414.066163923</v>
+        <v>1145706.187841673</v>
       </c>
       <c r="BW9" t="n">
-        <v>1515763.911566187</v>
+        <v>1027047.573270711</v>
       </c>
       <c r="BX9" t="n">
-        <v>1527797.363900427</v>
+        <v>1107606.637430847</v>
       </c>
       <c r="BY9" t="n">
-        <v>1382972.910274663</v>
+        <v>1026338.674711787</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: update tao's data format
</commit_message>
<xml_diff>
--- a/data/proteomics/protein_copy_statistical.xlsx
+++ b/data/proteomics/protein_copy_statistical.xlsx
@@ -425,63 +425,158 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:AE9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>maltose(mmol/gDW)</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>oleate(mmol/gDW)</t>
+          <t>S2</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>fructose(mmol/gDW)</t>
+          <t>S3</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>sucrose(mmol/gDW)</t>
+          <t>S4</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>trehalose(mmol/gDW)</t>
+          <t>S5</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>lactate(mmol/gDW)</t>
+          <t>S6</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>acetate(mmol/gDW)</t>
+          <t>S7</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>pryuvate(mmol/gDW)</t>
+          <t>S8</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>glycerol(mmol/gDW)</t>
+          <t>S9</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>galactose(mmol/gDW)</t>
+          <t>S10</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>raffinose(mmol/gDW)</t>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>S14</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>S15</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>S16</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>S17</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>S18</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>S19</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>S20</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>S21</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>S22</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>S23</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>S24</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>S25</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>S26</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>S27</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>S28</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>S29</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>S30</t>
         </is>
       </c>
     </row>
@@ -492,37 +587,94 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5003</v>
+        <v>2559</v>
       </c>
       <c r="C2" t="n">
-        <v>5003</v>
+        <v>2594</v>
       </c>
       <c r="D2" t="n">
-        <v>5003</v>
+        <v>2586</v>
       </c>
       <c r="E2" t="n">
-        <v>5003</v>
+        <v>2617</v>
       </c>
       <c r="F2" t="n">
-        <v>5003</v>
+        <v>2599</v>
       </c>
       <c r="G2" t="n">
-        <v>5003</v>
+        <v>2605</v>
       </c>
       <c r="H2" t="n">
-        <v>5003</v>
+        <v>2597</v>
       </c>
       <c r="I2" t="n">
-        <v>5003</v>
+        <v>2609</v>
       </c>
       <c r="J2" t="n">
-        <v>5003</v>
+        <v>2600</v>
       </c>
       <c r="K2" t="n">
-        <v>4675</v>
+        <v>2608</v>
       </c>
       <c r="L2" t="n">
-        <v>4675</v>
+        <v>2610</v>
+      </c>
+      <c r="M2" t="n">
+        <v>2586</v>
+      </c>
+      <c r="N2" t="n">
+        <v>2599</v>
+      </c>
+      <c r="O2" t="n">
+        <v>2614</v>
+      </c>
+      <c r="P2" t="n">
+        <v>2606</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>2608</v>
+      </c>
+      <c r="R2" t="n">
+        <v>2606</v>
+      </c>
+      <c r="S2" t="n">
+        <v>2603</v>
+      </c>
+      <c r="T2" t="n">
+        <v>2591</v>
+      </c>
+      <c r="U2" t="n">
+        <v>2587</v>
+      </c>
+      <c r="V2" t="n">
+        <v>2594</v>
+      </c>
+      <c r="W2" t="n">
+        <v>2613</v>
+      </c>
+      <c r="X2" t="n">
+        <v>2572</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>2604</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>2625</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>2627</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>2153</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>2616</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>2600</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>2607</v>
       </c>
     </row>
     <row r="3">
@@ -532,37 +684,94 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>18485.57923041054</v>
+        <v>21479.33653979915</v>
       </c>
       <c r="C3" t="n">
-        <v>19877.93171144229</v>
+        <v>21172.17586801982</v>
       </c>
       <c r="D3" t="n">
-        <v>19409.0015085981</v>
+        <v>21371.52902432103</v>
       </c>
       <c r="E3" t="n">
-        <v>19159.77728026655</v>
+        <v>20886.1582679575</v>
       </c>
       <c r="F3" t="n">
-        <v>18144.73355819078</v>
+        <v>20928.57155367203</v>
       </c>
       <c r="G3" t="n">
-        <v>18392.48050440425</v>
+        <v>21085.56719719686</v>
       </c>
       <c r="H3" t="n">
-        <v>22733.94674382204</v>
+        <v>20096.40808015182</v>
       </c>
       <c r="I3" t="n">
-        <v>20825.14545103406</v>
+        <v>19953.52490787723</v>
       </c>
       <c r="J3" t="n">
-        <v>19039.89691510175</v>
+        <v>19849.74846162785</v>
       </c>
       <c r="K3" t="n">
-        <v>17120.25161811963</v>
+        <v>19901.01008764332</v>
       </c>
       <c r="L3" t="n">
-        <v>16960.23272008139</v>
+        <v>19779.92607600213</v>
+      </c>
+      <c r="M3" t="n">
+        <v>19938.2394966369</v>
+      </c>
+      <c r="N3" t="n">
+        <v>19939.87020633948</v>
+      </c>
+      <c r="O3" t="n">
+        <v>19600.41347846734</v>
+      </c>
+      <c r="P3" t="n">
+        <v>19940.78699370214</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>19635.79476524408</v>
+      </c>
+      <c r="R3" t="n">
+        <v>19778.43757649073</v>
+      </c>
+      <c r="S3" t="n">
+        <v>19719.16472548874</v>
+      </c>
+      <c r="T3" t="n">
+        <v>20304.77230817149</v>
+      </c>
+      <c r="U3" t="n">
+        <v>20389.97748476532</v>
+      </c>
+      <c r="V3" t="n">
+        <v>20502.6322814846</v>
+      </c>
+      <c r="W3" t="n">
+        <v>20034.76709483627</v>
+      </c>
+      <c r="X3" t="n">
+        <v>20194.58092811797</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>20174.27171345919</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>19597.01931989633</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>19546.89319967055</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>23518.75027371082</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>19844.45115782679</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>19980.43172510442</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>20053.7610042189</v>
       </c>
     </row>
     <row r="4">
@@ -572,37 +781,94 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>111315.8457873329</v>
+        <v>89151.9004343507</v>
       </c>
       <c r="C4" t="n">
-        <v>121062.908847915</v>
+        <v>88502.74864847738</v>
       </c>
       <c r="D4" t="n">
-        <v>140739.2913885579</v>
+        <v>87926.75675522852</v>
       </c>
       <c r="E4" t="n">
-        <v>140222.1323186173</v>
+        <v>86632.32759835807</v>
       </c>
       <c r="F4" t="n">
-        <v>106428.738777524</v>
+        <v>87212.94621259523</v>
       </c>
       <c r="G4" t="n">
-        <v>106815.8881086667</v>
+        <v>87285.48422683335</v>
       </c>
       <c r="H4" t="n">
-        <v>145397.2715350767</v>
+        <v>85633.60541864428</v>
       </c>
       <c r="I4" t="n">
-        <v>140203.8699283449</v>
+        <v>84583.11315429914</v>
       </c>
       <c r="J4" t="n">
-        <v>112739.2075482871</v>
+        <v>84734.51977459206</v>
       </c>
       <c r="K4" t="n">
-        <v>136151.7548107124</v>
+        <v>84211.6243979651</v>
       </c>
       <c r="L4" t="n">
-        <v>122816.8832387086</v>
+        <v>84473.00928802532</v>
+      </c>
+      <c r="M4" t="n">
+        <v>84461.31234689032</v>
+      </c>
+      <c r="N4" t="n">
+        <v>85042.59710339077</v>
+      </c>
+      <c r="O4" t="n">
+        <v>83644.7614051873</v>
+      </c>
+      <c r="P4" t="n">
+        <v>85172.15242561299</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>83796.95271283206</v>
+      </c>
+      <c r="R4" t="n">
+        <v>84421.17049699005</v>
+      </c>
+      <c r="S4" t="n">
+        <v>83550.6954379924</v>
+      </c>
+      <c r="T4" t="n">
+        <v>86972.50935426423</v>
+      </c>
+      <c r="U4" t="n">
+        <v>86890.15384032724</v>
+      </c>
+      <c r="V4" t="n">
+        <v>87499.43015570736</v>
+      </c>
+      <c r="W4" t="n">
+        <v>86719.86810228477</v>
+      </c>
+      <c r="X4" t="n">
+        <v>87523.99444919142</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>88289.39814433924</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>84593.34102847974</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>84164.68819306923</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>93089.19466040657</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>84491.27937109229</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>84754.65224824105</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>85383.4442641178</v>
       </c>
     </row>
     <row r="5">
@@ -612,37 +878,94 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>0.7380148598524247</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>0.6666135591110226</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>1.310357515392214</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>0.6603285993948841</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>0.8882790443124121</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>0.2098137979542027</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>0.2597074223230679</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>0.3695729241777767</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>0.3506733767350964</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>0.6224724706795639</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>0.3009405786470385</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.6118399747471337</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.1744441069980964</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.5073285349721516</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.3543997651972595</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0.67545207916949</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0.5740195477613695</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0.5152724677507932</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0.5604648312208235</v>
+      </c>
+      <c r="U5" t="n">
+        <v>1.689014949807587</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.6099683043929417</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0.6024476431161023</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0.8267622131534704</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>0.5754901477640921</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>0.4455368948512177</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>0.7352106967330879</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>0.5826920627495892</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>0.1090882774587115</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>0.6728682593666947</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>0.9413104979674254</v>
       </c>
     </row>
     <row r="6">
@@ -652,37 +975,94 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>321.2429025725583</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>310.4380847101929</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>316.6765958954319</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>306.1529324141288</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>312.1786505290289</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>294.8954402908781</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>321.3026663162254</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>304.2363906189938</v>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>319.2456858612654</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>292.2159952678215</v>
       </c>
       <c r="L6" t="n">
-        <v>0</v>
+        <v>321.6186508120586</v>
+      </c>
+      <c r="M6" t="n">
+        <v>325.9829867095046</v>
+      </c>
+      <c r="N6" t="n">
+        <v>322.4241213239002</v>
+      </c>
+      <c r="O6" t="n">
+        <v>326.4011271478557</v>
+      </c>
+      <c r="P6" t="n">
+        <v>323.6035060162353</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>327.387842185422</v>
+      </c>
+      <c r="R6" t="n">
+        <v>311.7128893397294</v>
+      </c>
+      <c r="S6" t="n">
+        <v>333.0602715278042</v>
+      </c>
+      <c r="T6" t="n">
+        <v>325.5584364834521</v>
+      </c>
+      <c r="U6" t="n">
+        <v>310.9937028522037</v>
+      </c>
+      <c r="V6" t="n">
+        <v>311.5261015244307</v>
+      </c>
+      <c r="W6" t="n">
+        <v>315.8026378178911</v>
+      </c>
+      <c r="X6" t="n">
+        <v>330.6731741106112</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>294.8077245843033</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>308.4200894322775</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>303.5729540078164</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>435.7573601181748</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>313.2972610180983</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>307.0462478137434</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>302.8073581785844</v>
       </c>
     </row>
     <row r="7">
@@ -692,37 +1072,94 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>324.6317986632183</v>
+        <v>1255.636401589482</v>
       </c>
       <c r="C7" t="n">
-        <v>350.1456340418788</v>
+        <v>1252.688493255059</v>
       </c>
       <c r="D7" t="n">
-        <v>370.9677987451415</v>
+        <v>1276.175594368195</v>
       </c>
       <c r="E7" t="n">
-        <v>377.6731503940441</v>
+        <v>1234.63856524325</v>
       </c>
       <c r="F7" t="n">
-        <v>353.6707032642191</v>
+        <v>1213.505279244668</v>
       </c>
       <c r="G7" t="n">
-        <v>364.8590157232369</v>
+        <v>1220.23917968537</v>
       </c>
       <c r="H7" t="n">
-        <v>339.2015691032469</v>
+        <v>1213.572939953293</v>
       </c>
       <c r="I7" t="n">
-        <v>392.5928287176063</v>
+        <v>1211.633456930948</v>
       </c>
       <c r="J7" t="n">
-        <v>387.7875861359022</v>
+        <v>1229.183211732243</v>
       </c>
       <c r="K7" t="n">
-        <v>532.1152826546157</v>
+        <v>1201.006837742072</v>
       </c>
       <c r="L7" t="n">
-        <v>486.2243460482219</v>
+        <v>1228.514466806443</v>
+      </c>
+      <c r="M7" t="n">
+        <v>1236.701651452297</v>
+      </c>
+      <c r="N7" t="n">
+        <v>1203.782788373285</v>
+      </c>
+      <c r="O7" t="n">
+        <v>1230.531947083542</v>
+      </c>
+      <c r="P7" t="n">
+        <v>1217.626235120937</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>1185.135527130219</v>
+      </c>
+      <c r="R7" t="n">
+        <v>1212.301187623168</v>
+      </c>
+      <c r="S7" t="n">
+        <v>1197.066122920919</v>
+      </c>
+      <c r="T7" t="n">
+        <v>1214.879219773978</v>
+      </c>
+      <c r="U7" t="n">
+        <v>1213.814704720891</v>
+      </c>
+      <c r="V7" t="n">
+        <v>1188.829048445776</v>
+      </c>
+      <c r="W7" t="n">
+        <v>1200.173747939396</v>
+      </c>
+      <c r="X7" t="n">
+        <v>1218.359615188093</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>1193.399680497446</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>1154.261758521151</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>1183.148236431594</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>1684.106299541941</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>1176.576326855899</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>1188.849601399891</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>1206.722640819842</v>
       </c>
     </row>
     <row r="8">
@@ -732,37 +1169,94 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2714.763019572504</v>
+        <v>5559.598039072929</v>
       </c>
       <c r="C8" t="n">
-        <v>2936.210470480949</v>
+        <v>5443.192618634062</v>
       </c>
       <c r="D8" t="n">
-        <v>2999.314310180298</v>
+        <v>5737.369921467342</v>
       </c>
       <c r="E8" t="n">
-        <v>3111.551629923011</v>
+        <v>5564.451035711741</v>
       </c>
       <c r="F8" t="n">
-        <v>3002.571606630671</v>
+        <v>5544.107707887068</v>
       </c>
       <c r="G8" t="n">
-        <v>3003.576668248743</v>
+        <v>5483.96080859617</v>
       </c>
       <c r="H8" t="n">
-        <v>2876.622574639217</v>
+        <v>5563.985295366831</v>
       </c>
       <c r="I8" t="n">
-        <v>3230.32160578173</v>
+        <v>5458.880453932423</v>
       </c>
       <c r="J8" t="n">
-        <v>3245.43340987828</v>
+        <v>5472.162861727676</v>
       </c>
       <c r="K8" t="n">
-        <v>3418.42180444752</v>
+        <v>5459.398192667587</v>
       </c>
       <c r="L8" t="n">
-        <v>3241.058766830559</v>
+        <v>5486.079588157132</v>
+      </c>
+      <c r="M8" t="n">
+        <v>5523.770351357613</v>
+      </c>
+      <c r="N8" t="n">
+        <v>5610.296902595914</v>
+      </c>
+      <c r="O8" t="n">
+        <v>5529.910547059703</v>
+      </c>
+      <c r="P8" t="n">
+        <v>5400.720115933402</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>5274.651706699782</v>
+      </c>
+      <c r="R8" t="n">
+        <v>5503.758524167823</v>
+      </c>
+      <c r="S8" t="n">
+        <v>5515.442072197141</v>
+      </c>
+      <c r="T8" t="n">
+        <v>5468.856333913383</v>
+      </c>
+      <c r="U8" t="n">
+        <v>5425.627142181072</v>
+      </c>
+      <c r="V8" t="n">
+        <v>5548.452594999504</v>
+      </c>
+      <c r="W8" t="n">
+        <v>5374.991239151143</v>
+      </c>
+      <c r="X8" t="n">
+        <v>5423.475387721582</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>5405.869342909304</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>5306.644516907553</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>5478.297835677508</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>7576.892042329007</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>5478.4234575265</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>5534.428692330821</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>5526.743010984213</v>
       </c>
     </row>
     <row r="9">
@@ -772,37 +1266,94 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3441293.778590984</v>
+        <v>1943049.664115919</v>
       </c>
       <c r="C9" t="n">
-        <v>2997519.452074238</v>
+        <v>1983105.574626185</v>
       </c>
       <c r="D9" t="n">
-        <v>3474572.365462308</v>
+        <v>1914430.095727566</v>
       </c>
       <c r="E9" t="n">
-        <v>3766905.59001234</v>
+        <v>1945154.819028278</v>
       </c>
       <c r="F9" t="n">
-        <v>2753403.630072502</v>
+        <v>1998587.776671322</v>
       </c>
       <c r="G9" t="n">
-        <v>2173211.290130805</v>
+        <v>1918674.373789614</v>
       </c>
       <c r="H9" t="n">
-        <v>3039979.376189653</v>
+        <v>2137465.011001145</v>
       </c>
       <c r="I9" t="n">
-        <v>6004868.809911354</v>
+        <v>2124551.042110998</v>
       </c>
       <c r="J9" t="n">
-        <v>2247437.265527637</v>
+        <v>2151800.826652864</v>
       </c>
       <c r="K9" t="n">
-        <v>5375654.536827597</v>
+        <v>2105580.175655238</v>
       </c>
       <c r="L9" t="n">
-        <v>4239740.357313359</v>
+        <v>2171133.869241349</v>
+      </c>
+      <c r="M9" t="n">
+        <v>2100201.602780261</v>
+      </c>
+      <c r="N9" t="n">
+        <v>2169433.580600113</v>
+      </c>
+      <c r="O9" t="n">
+        <v>2150009.559917057</v>
+      </c>
+      <c r="P9" t="n">
+        <v>2200059.489675947</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>2112649.063402391</v>
+      </c>
+      <c r="R9" t="n">
+        <v>2130198.594493009</v>
+      </c>
+      <c r="S9" t="n">
+        <v>2132771.306836835</v>
+      </c>
+      <c r="T9" t="n">
+        <v>2192154.428067199</v>
+      </c>
+      <c r="U9" t="n">
+        <v>2172264.044427255</v>
+      </c>
+      <c r="V9" t="n">
+        <v>2155059.709455179</v>
+      </c>
+      <c r="W9" t="n">
+        <v>2208836.99664789</v>
+      </c>
+      <c r="X9" t="n">
+        <v>2263723.472387413</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>2363332.081626541</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>2209963.484593864</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>2183302.056370241</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>2173948.79615762</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>2093456.443268903</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>2121380.719582611</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>2165432.92409642</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: update figure code
</commit_message>
<xml_diff>
--- a/data/proteomics/protein_copy_statistical.xlsx
+++ b/data/proteomics/protein_copy_statistical.xlsx
@@ -425,63 +425,388 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:BY9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>maltose(mmol/gDW)</t>
+          <t>Glucose_phase(mmol/gDW)</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>oleate(mmol/gDW)</t>
+          <t>Diauxic_shift(mmol/gDW)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>fructose(mmol/gDW)</t>
+          <t>Ethanol_phase(mmol/gDW)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>sucrose(mmol/gDW)</t>
+          <t>mmol/gDW_carl</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>trehalose(mmol/gDW)</t>
+          <t>prot.1</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>lactate(mmol/gDW)</t>
+          <t>prot.10</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>acetate(mmol/gDW)</t>
+          <t>prot.11</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>pryuvate(mmol/gDW)</t>
+          <t>prot.12</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>glycerol(mmol/gDW)</t>
+          <t>prot.13</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>galactose(mmol/gDW)</t>
+          <t>prot.14</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>raffinose(mmol/gDW)</t>
+          <t>prot.15</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>prot.16</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>prot.17</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>prot.18</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>prot.19</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>prot.2</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>prot.20</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>prot.21</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>prot.22</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>prot.23</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>prot.24</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>prot.25</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>prot.26</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>prot.27</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>prot.28</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>prot.29</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>prot.3</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>prot.30</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>prot.31</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>prot.32</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>prot.33</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>prot.34</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>prot.35</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>prot.36</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>prot.37</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>prot.38</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>prot.39</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>prot.4</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>prot.40</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>prot.41</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>prot.42</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>prot.5</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>prot.6</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>prot.7</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>prot.8</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>prot.9</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>mmol/gDW_Tyler_D0.1</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>Min_ave_aerobic(mmol/gDW)</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>Rich_ave_aerobic(mmol/gDW)</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>Min_ave_anaerobic(mmol/gDW)</t>
+        </is>
+      </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>Rich_ave_anaerobic(mmol/gDW)</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>mean_REF_CN4_D=0.1</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>mean_CN22_D=0.1</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>mean_CN38_D=0.1</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>mean_CN75_D=0.1</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>FG_rep1_CN4_D= 0.26 or 0.32</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>FG_rep2_CN4_D= 0.26 or 0.32</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>FG_rep3_CN4_D= 0.26 or 0.32</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>FG_rep4_CN4_D= 0.26 or 0.32</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>molecular/cell_paxdb</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ghaemmaghami et al. 2003 - Copy </t>
+        </is>
+      </c>
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>Kulak et al. 2014 - Copy</t>
+        </is>
+      </c>
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
+          <t>Mean Copy number - Glucose</t>
+        </is>
+      </c>
+      <c r="BM1" s="1" t="inlineStr">
+        <is>
+          <t>Mean Copy number - Galactose</t>
+        </is>
+      </c>
+      <c r="BN1" s="1" t="inlineStr">
+        <is>
+          <t>Mean Copy number - Glycerol</t>
+        </is>
+      </c>
+      <c r="BO1" s="1" t="inlineStr">
+        <is>
+          <t>Mean molecules per cell_cell_system_2018</t>
+        </is>
+      </c>
+      <c r="BP1" s="1" t="inlineStr">
+        <is>
+          <t>Median molecules per cell_cell_system_2018</t>
+        </is>
+      </c>
+      <c r="BQ1" s="1" t="inlineStr">
+        <is>
+          <t>D=0.027_M</t>
+        </is>
+      </c>
+      <c r="BR1" s="1" t="inlineStr">
+        <is>
+          <t>D=0.044_M</t>
+        </is>
+      </c>
+      <c r="BS1" s="1" t="inlineStr">
+        <is>
+          <t>D=0.102_M</t>
+        </is>
+      </c>
+      <c r="BT1" s="1" t="inlineStr">
+        <is>
+          <t>D=0.152_M</t>
+        </is>
+      </c>
+      <c r="BU1" s="1" t="inlineStr">
+        <is>
+          <t>D=0.214_M</t>
+        </is>
+      </c>
+      <c r="BV1" s="1" t="inlineStr">
+        <is>
+          <t>D=0.254_M</t>
+        </is>
+      </c>
+      <c r="BW1" s="1" t="inlineStr">
+        <is>
+          <t>D=0.284_M</t>
+        </is>
+      </c>
+      <c r="BX1" s="1" t="inlineStr">
+        <is>
+          <t>D=0.334_M</t>
+        </is>
+      </c>
+      <c r="BY1" s="1" t="inlineStr">
+        <is>
+          <t>D=0.379_M</t>
         </is>
       </c>
     </row>
@@ -492,37 +817,232 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5003</v>
+        <v>3801</v>
       </c>
       <c r="C2" t="n">
-        <v>5003</v>
+        <v>3802</v>
       </c>
       <c r="D2" t="n">
-        <v>5003</v>
+        <v>3802</v>
       </c>
       <c r="E2" t="n">
-        <v>5003</v>
+        <v>3928</v>
       </c>
       <c r="F2" t="n">
-        <v>5003</v>
+        <v>3128</v>
       </c>
       <c r="G2" t="n">
-        <v>5003</v>
+        <v>3128</v>
       </c>
       <c r="H2" t="n">
-        <v>5003</v>
+        <v>3128</v>
       </c>
       <c r="I2" t="n">
-        <v>5003</v>
+        <v>3128</v>
       </c>
       <c r="J2" t="n">
-        <v>5003</v>
+        <v>3128</v>
       </c>
       <c r="K2" t="n">
-        <v>4675</v>
+        <v>3128</v>
       </c>
       <c r="L2" t="n">
-        <v>4675</v>
+        <v>3128</v>
+      </c>
+      <c r="M2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="N2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="O2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="P2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="R2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="S2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="T2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="U2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="V2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="W2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="X2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="AP2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="AU2" t="n">
+        <v>3128</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>2142</v>
+      </c>
+      <c r="AW2" t="n">
+        <v>3690</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>3690</v>
+      </c>
+      <c r="AY2" t="n">
+        <v>3690</v>
+      </c>
+      <c r="AZ2" t="n">
+        <v>3690</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>2634</v>
+      </c>
+      <c r="BB2" t="n">
+        <v>2628</v>
+      </c>
+      <c r="BC2" t="n">
+        <v>2657</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>2646</v>
+      </c>
+      <c r="BE2" t="n">
+        <v>2308</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>2327</v>
+      </c>
+      <c r="BG2" t="n">
+        <v>2331</v>
+      </c>
+      <c r="BH2" t="n">
+        <v>2359</v>
+      </c>
+      <c r="BI2" t="n">
+        <v>6440</v>
+      </c>
+      <c r="BJ2" t="n">
+        <v>3868</v>
+      </c>
+      <c r="BK2" t="n">
+        <v>4636</v>
+      </c>
+      <c r="BL2" t="n">
+        <v>4148</v>
+      </c>
+      <c r="BM2" t="n">
+        <v>4148</v>
+      </c>
+      <c r="BN2" t="n">
+        <v>4148</v>
+      </c>
+      <c r="BO2" t="n">
+        <v>5391</v>
+      </c>
+      <c r="BP2" t="n">
+        <v>5391</v>
+      </c>
+      <c r="BQ2" t="n">
+        <v>2561</v>
+      </c>
+      <c r="BR2" t="n">
+        <v>2525</v>
+      </c>
+      <c r="BS2" t="n">
+        <v>2512</v>
+      </c>
+      <c r="BT2" t="n">
+        <v>2469</v>
+      </c>
+      <c r="BU2" t="n">
+        <v>2490</v>
+      </c>
+      <c r="BV2" t="n">
+        <v>2473</v>
+      </c>
+      <c r="BW2" t="n">
+        <v>2526</v>
+      </c>
+      <c r="BX2" t="n">
+        <v>2438</v>
+      </c>
+      <c r="BY2" t="n">
+        <v>2421</v>
       </c>
     </row>
     <row r="3">
@@ -532,37 +1052,232 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>18485.57923041054</v>
+        <v>31699.93008138769</v>
       </c>
       <c r="C3" t="n">
-        <v>19877.93171144229</v>
+        <v>28687.47638216143</v>
       </c>
       <c r="D3" t="n">
-        <v>19409.0015085981</v>
+        <v>25039.36838391844</v>
       </c>
       <c r="E3" t="n">
-        <v>19159.77728026655</v>
+        <v>27809.26232010378</v>
       </c>
       <c r="F3" t="n">
-        <v>18144.73355819078</v>
+        <v>12518.42934284728</v>
       </c>
       <c r="G3" t="n">
-        <v>18392.48050440425</v>
+        <v>14073.40599052339</v>
       </c>
       <c r="H3" t="n">
-        <v>22733.94674382204</v>
+        <v>12038.61901122389</v>
       </c>
       <c r="I3" t="n">
-        <v>20825.14545103406</v>
+        <v>12049.98975133031</v>
       </c>
       <c r="J3" t="n">
-        <v>19039.89691510175</v>
+        <v>13278.63061451924</v>
       </c>
       <c r="K3" t="n">
-        <v>17120.25161811963</v>
+        <v>12955.02173001969</v>
       </c>
       <c r="L3" t="n">
-        <v>16960.23272008139</v>
+        <v>13073.89329933087</v>
+      </c>
+      <c r="M3" t="n">
+        <v>22101.55608720983</v>
+      </c>
+      <c r="N3" t="n">
+        <v>22145.20565946272</v>
+      </c>
+      <c r="O3" t="n">
+        <v>20929.35619261183</v>
+      </c>
+      <c r="P3" t="n">
+        <v>27481.03484670626</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>11273.41152578673</v>
+      </c>
+      <c r="R3" t="n">
+        <v>29003.88583055399</v>
+      </c>
+      <c r="S3" t="n">
+        <v>28923.62587780414</v>
+      </c>
+      <c r="T3" t="n">
+        <v>24828.64835487205</v>
+      </c>
+      <c r="U3" t="n">
+        <v>30025.26094565109</v>
+      </c>
+      <c r="V3" t="n">
+        <v>30818.38815773577</v>
+      </c>
+      <c r="W3" t="n">
+        <v>23716.62980526402</v>
+      </c>
+      <c r="X3" t="n">
+        <v>13994.52970436225</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>17422.97033576227</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>10019.73321055387</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>16401.9036189057</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>12067.89495158295</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>16291.49478922326</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>18880.99950768716</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>23471.27299244677</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>20160.17033812535</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>18998.38899176757</v>
+      </c>
+      <c r="AH3" t="n">
+        <v>17108.93412808232</v>
+      </c>
+      <c r="AI3" t="n">
+        <v>18038.95622030722</v>
+      </c>
+      <c r="AJ3" t="n">
+        <v>14969.74580855612</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>19545.68585555418</v>
+      </c>
+      <c r="AL3" t="n">
+        <v>16673.01648769615</v>
+      </c>
+      <c r="AM3" t="n">
+        <v>17883.05462836951</v>
+      </c>
+      <c r="AN3" t="n">
+        <v>22750.91520827561</v>
+      </c>
+      <c r="AO3" t="n">
+        <v>21842.0061224755</v>
+      </c>
+      <c r="AP3" t="n">
+        <v>21217.03775782351</v>
+      </c>
+      <c r="AQ3" t="n">
+        <v>19079.54603901364</v>
+      </c>
+      <c r="AR3" t="n">
+        <v>16074.75695563478</v>
+      </c>
+      <c r="AS3" t="n">
+        <v>9304.260545395471</v>
+      </c>
+      <c r="AT3" t="n">
+        <v>9827.985033674569</v>
+      </c>
+      <c r="AU3" t="n">
+        <v>12951.24194404544</v>
+      </c>
+      <c r="AV3" t="n">
+        <v>26692.50099691877</v>
+      </c>
+      <c r="AW3" t="n">
+        <v>30739.82382791224</v>
+      </c>
+      <c r="AX3" t="n">
+        <v>31699.64696088852</v>
+      </c>
+      <c r="AY3" t="n">
+        <v>27174.0003533339</v>
+      </c>
+      <c r="AZ3" t="n">
+        <v>28318.70378302562</v>
+      </c>
+      <c r="BA3" t="n">
+        <v>47527.29071438549</v>
+      </c>
+      <c r="BB3" t="n">
+        <v>30113.65362905579</v>
+      </c>
+      <c r="BC3" t="n">
+        <v>47748.0810349111</v>
+      </c>
+      <c r="BD3" t="n">
+        <v>24569.76996107538</v>
+      </c>
+      <c r="BE3" t="n">
+        <v>37948.10186016465</v>
+      </c>
+      <c r="BF3" t="n">
+        <v>36985.03807516381</v>
+      </c>
+      <c r="BG3" t="n">
+        <v>38421.47544668819</v>
+      </c>
+      <c r="BH3" t="n">
+        <v>37157.29537987077</v>
+      </c>
+      <c r="BI3" t="n">
+        <v>12422.29275776397</v>
+      </c>
+      <c r="BJ3" t="n">
+        <v>12064.23767219401</v>
+      </c>
+      <c r="BK3" t="n">
+        <v>11685.94367859411</v>
+      </c>
+      <c r="BL3" t="n">
+        <v>15277.96070395371</v>
+      </c>
+      <c r="BM3" t="n">
+        <v>11837.10390549662</v>
+      </c>
+      <c r="BN3" t="n">
+        <v>14464.3743972999</v>
+      </c>
+      <c r="BO3" t="n">
+        <v>11388.10700346718</v>
+      </c>
+      <c r="BP3" t="n">
+        <v>7764.094734708288</v>
+      </c>
+      <c r="BQ3" t="n">
+        <v>29011.57474618037</v>
+      </c>
+      <c r="BR3" t="n">
+        <v>30262.65525463245</v>
+      </c>
+      <c r="BS3" t="n">
+        <v>33453.28722159965</v>
+      </c>
+      <c r="BT3" t="n">
+        <v>37288.8691853261</v>
+      </c>
+      <c r="BU3" t="n">
+        <v>27388.1535813967</v>
+      </c>
+      <c r="BV3" t="n">
+        <v>31889.76673746826</v>
+      </c>
+      <c r="BW3" t="n">
+        <v>32153.46160666694</v>
+      </c>
+      <c r="BX3" t="n">
+        <v>34480.69774000028</v>
+      </c>
+      <c r="BY3" t="n">
+        <v>31284.70605537057</v>
       </c>
     </row>
     <row r="4">
@@ -572,37 +1287,232 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>111315.8457873329</v>
+        <v>248305.7799069178</v>
       </c>
       <c r="C4" t="n">
-        <v>121062.908847915</v>
+        <v>155392.3952094483</v>
       </c>
       <c r="D4" t="n">
-        <v>140739.2913885579</v>
+        <v>154715.8728319417</v>
       </c>
       <c r="E4" t="n">
-        <v>140222.1323186173</v>
+        <v>141223.2894959995</v>
       </c>
       <c r="F4" t="n">
-        <v>106428.738777524</v>
+        <v>66918.75512960671</v>
       </c>
       <c r="G4" t="n">
-        <v>106815.8881086667</v>
+        <v>71709.43327629076</v>
       </c>
       <c r="H4" t="n">
-        <v>145397.2715350767</v>
+        <v>63891.0400374174</v>
       </c>
       <c r="I4" t="n">
-        <v>140203.8699283449</v>
+        <v>62268.56123348384</v>
       </c>
       <c r="J4" t="n">
-        <v>112739.2075482871</v>
+        <v>65786.07688594142</v>
       </c>
       <c r="K4" t="n">
-        <v>136151.7548107124</v>
+        <v>64565.5174438578</v>
       </c>
       <c r="L4" t="n">
-        <v>122816.8832387086</v>
+        <v>68284.49105461262</v>
+      </c>
+      <c r="M4" t="n">
+        <v>116896.4757637392</v>
+      </c>
+      <c r="N4" t="n">
+        <v>114124.7746417368</v>
+      </c>
+      <c r="O4" t="n">
+        <v>106860.0609547023</v>
+      </c>
+      <c r="P4" t="n">
+        <v>142647.5166379431</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>60518.16560546382</v>
+      </c>
+      <c r="R4" t="n">
+        <v>153554.5969986021</v>
+      </c>
+      <c r="S4" t="n">
+        <v>149557.2542187138</v>
+      </c>
+      <c r="T4" t="n">
+        <v>175499.2435029291</v>
+      </c>
+      <c r="U4" t="n">
+        <v>207095.757270361</v>
+      </c>
+      <c r="V4" t="n">
+        <v>207590.2535045513</v>
+      </c>
+      <c r="W4" t="n">
+        <v>134082.8838197027</v>
+      </c>
+      <c r="X4" t="n">
+        <v>75151.72501234972</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>96112.14596625253</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>49828.48776493017</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>81158.16824771844</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>67819.35466305827</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>80526.3478628739</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>103059.9498914771</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>135538.6127013691</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>109537.1553925181</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>100658.6485246631</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>86439.74708679192</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>89448.19028639616</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>82218.62331929988</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>113109.3165817835</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>90413.41583845747</v>
+      </c>
+      <c r="AM4" t="n">
+        <v>112992.8999783003</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>118705.3108374197</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>116894.1264883224</v>
+      </c>
+      <c r="AP4" t="n">
+        <v>113008.3704132263</v>
+      </c>
+      <c r="AQ4" t="n">
+        <v>123906.1068952232</v>
+      </c>
+      <c r="AR4" t="n">
+        <v>96366.74830504799</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>51483.08474887283</v>
+      </c>
+      <c r="AT4" t="n">
+        <v>53737.12567912344</v>
+      </c>
+      <c r="AU4" t="n">
+        <v>68154.49267078238</v>
+      </c>
+      <c r="AV4" t="n">
+        <v>84421.98038418527</v>
+      </c>
+      <c r="AW4" t="n">
+        <v>175075.6849168531</v>
+      </c>
+      <c r="AX4" t="n">
+        <v>184892.4862760086</v>
+      </c>
+      <c r="AY4" t="n">
+        <v>182528.7240083382</v>
+      </c>
+      <c r="AZ4" t="n">
+        <v>189211.8200729666</v>
+      </c>
+      <c r="BA4" t="n">
+        <v>194937.7146462307</v>
+      </c>
+      <c r="BB4" t="n">
+        <v>116480.6872823338</v>
+      </c>
+      <c r="BC4" t="n">
+        <v>191407.9031324337</v>
+      </c>
+      <c r="BD4" t="n">
+        <v>95665.31281119701</v>
+      </c>
+      <c r="BE4" t="n">
+        <v>137212.9599842691</v>
+      </c>
+      <c r="BF4" t="n">
+        <v>133747.8429605585</v>
+      </c>
+      <c r="BG4" t="n">
+        <v>138499.505557799</v>
+      </c>
+      <c r="BH4" t="n">
+        <v>134072.9752590545</v>
+      </c>
+      <c r="BI4" t="n">
+        <v>56887.47554446503</v>
+      </c>
+      <c r="BJ4" t="n">
+        <v>55802.48951649197</v>
+      </c>
+      <c r="BK4" t="n">
+        <v>50249.86452774274</v>
+      </c>
+      <c r="BL4" t="n">
+        <v>69811.37557685096</v>
+      </c>
+      <c r="BM4" t="n">
+        <v>47863.20519554242</v>
+      </c>
+      <c r="BN4" t="n">
+        <v>61678.22098880803</v>
+      </c>
+      <c r="BO4" t="n">
+        <v>48612.96283046022</v>
+      </c>
+      <c r="BP4" t="n">
+        <v>27505.07111669971</v>
+      </c>
+      <c r="BQ4" t="n">
+        <v>119518.5718200878</v>
+      </c>
+      <c r="BR4" t="n">
+        <v>115424.9224959265</v>
+      </c>
+      <c r="BS4" t="n">
+        <v>99572.66923928485</v>
+      </c>
+      <c r="BT4" t="n">
+        <v>100702.5203317217</v>
+      </c>
+      <c r="BU4" t="n">
+        <v>70673.84324781052</v>
+      </c>
+      <c r="BV4" t="n">
+        <v>82860.57921750014</v>
+      </c>
+      <c r="BW4" t="n">
+        <v>83422.5148094544</v>
+      </c>
+      <c r="BX4" t="n">
+        <v>89262.80278051979</v>
+      </c>
+      <c r="BY4" t="n">
+        <v>82206.88924311596</v>
       </c>
     </row>
     <row r="5">
@@ -612,16 +1522,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>0.3331524685671092</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>0.6869436788094998</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>0.8963844210861369</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>11.30615094046392</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -643,6 +1553,201 @@
       </c>
       <c r="L5" t="n">
         <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA5" t="n">
+        <v>2.950007664697639</v>
+      </c>
+      <c r="BB5" t="n">
+        <v>1.377207742898766</v>
+      </c>
+      <c r="BC5" t="n">
+        <v>2.2053526682482</v>
+      </c>
+      <c r="BD5" t="n">
+        <v>1.449799280300976</v>
+      </c>
+      <c r="BE5" t="n">
+        <v>0.9270381111036474</v>
+      </c>
+      <c r="BF5" t="n">
+        <v>0.887305381384657</v>
+      </c>
+      <c r="BG5" t="n">
+        <v>9.563797890416424</v>
+      </c>
+      <c r="BH5" t="n">
+        <v>0.9166766157201268</v>
+      </c>
+      <c r="BI5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ5" t="n">
+        <v>41.1</v>
+      </c>
+      <c r="BK5" t="n">
+        <v>0.6786894999999999</v>
+      </c>
+      <c r="BL5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO5" t="n">
+        <v>3.359783478</v>
+      </c>
+      <c r="BP5" t="n">
+        <v>3.359783478</v>
+      </c>
+      <c r="BQ5" t="n">
+        <v>7.81185571641712</v>
+      </c>
+      <c r="BR5" t="n">
+        <v>15.45839164554615</v>
+      </c>
+      <c r="BS5" t="n">
+        <v>6.05724045057285</v>
+      </c>
+      <c r="BT5" t="n">
+        <v>9.93604934402661</v>
+      </c>
+      <c r="BU5" t="n">
+        <v>7.40295805265724</v>
+      </c>
+      <c r="BV5" t="n">
+        <v>12.9261462771642</v>
+      </c>
+      <c r="BW5" t="n">
+        <v>7.39889935614877</v>
+      </c>
+      <c r="BX5" t="n">
+        <v>10.6923993930067</v>
+      </c>
+      <c r="BY5" t="n">
+        <v>10.408059734663</v>
       </c>
     </row>
     <row r="6">
@@ -652,37 +1757,232 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>167.9689704545565</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>223.4463347942532</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>229.1642297708295</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>598.8225460547256</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>80.153840101566</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>89.22383774915599</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>75.04330767897702</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>78.29737540315185</v>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>87.24983850770549</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>84.6444452708525</v>
       </c>
       <c r="L6" t="n">
-        <v>0</v>
+        <v>86.74419417349949</v>
+      </c>
+      <c r="M6" t="n">
+        <v>116.063392636037</v>
+      </c>
+      <c r="N6" t="n">
+        <v>122.228649425091</v>
+      </c>
+      <c r="O6" t="n">
+        <v>113.495998162415</v>
+      </c>
+      <c r="P6" t="n">
+        <v>126.504210566316</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>71.92754186199616</v>
+      </c>
+      <c r="R6" t="n">
+        <v>124.7542174007305</v>
+      </c>
+      <c r="S6" t="n">
+        <v>132.988979687377</v>
+      </c>
+      <c r="T6" t="n">
+        <v>129.9786733350215</v>
+      </c>
+      <c r="U6" t="n">
+        <v>149.069780098371</v>
+      </c>
+      <c r="V6" t="n">
+        <v>150.3660340050165</v>
+      </c>
+      <c r="W6" t="n">
+        <v>131.6739927493375</v>
+      </c>
+      <c r="X6" t="n">
+        <v>79.3925757582485</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>97.94365716367651</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>57.02712346285405</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>97.682689048824</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>72.25688582135211</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>101.874785070135</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>115.6961743309295</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>132.0487719595385</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>116.195795571911</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>127.8639982888895</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>109.2292227418975</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>113.1034768798825</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>93.56920149865749</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>118.2239190105435</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>92.42240277526301</v>
+      </c>
+      <c r="AM6" t="n">
+        <v>101.349335335127</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>115.4205619258175</v>
+      </c>
+      <c r="AO6" t="n">
+        <v>123.6904722433875</v>
+      </c>
+      <c r="AP6" t="n">
+        <v>114.9420963933715</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>102.1709409717205</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>88.87837446505051</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>60.94255695019196</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>64.34762314643191</v>
+      </c>
+      <c r="AU6" t="n">
+        <v>68.32148353311601</v>
+      </c>
+      <c r="AV6" t="n">
+        <v>276.1309466666666</v>
+      </c>
+      <c r="AW6" t="n">
+        <v>199.6209220702642</v>
+      </c>
+      <c r="AX6" t="n">
+        <v>217.5880158156825</v>
+      </c>
+      <c r="AY6" t="n">
+        <v>233.1055674764273</v>
+      </c>
+      <c r="AZ6" t="n">
+        <v>253.2547174155409</v>
+      </c>
+      <c r="BA6" t="n">
+        <v>1459.815858569299</v>
+      </c>
+      <c r="BB6" t="n">
+        <v>1010.238493326309</v>
+      </c>
+      <c r="BC6" t="n">
+        <v>1479.679414962318</v>
+      </c>
+      <c r="BD6" t="n">
+        <v>793.0391721131303</v>
+      </c>
+      <c r="BE6" t="n">
+        <v>1391.618469735625</v>
+      </c>
+      <c r="BF6" t="n">
+        <v>1302.921624880578</v>
+      </c>
+      <c r="BG6" t="n">
+        <v>1375.226008848034</v>
+      </c>
+      <c r="BH6" t="n">
+        <v>1354.791949708646</v>
+      </c>
+      <c r="BI6" t="n">
+        <v>196.8</v>
+      </c>
+      <c r="BJ6" t="n">
+        <v>876.399693536828</v>
+      </c>
+      <c r="BK6" t="n">
+        <v>188.1809</v>
+      </c>
+      <c r="BL6" t="n">
+        <v>230</v>
+      </c>
+      <c r="BM6" t="n">
+        <v>183</v>
+      </c>
+      <c r="BN6" t="n">
+        <v>232.75</v>
+      </c>
+      <c r="BO6" t="n">
+        <v>1579.20900869</v>
+      </c>
+      <c r="BP6" t="n">
+        <v>1391.58692875209</v>
+      </c>
+      <c r="BQ6" t="n">
+        <v>1260.80884481044</v>
+      </c>
+      <c r="BR6" t="n">
+        <v>1381.107826577527</v>
+      </c>
+      <c r="BS6" t="n">
+        <v>1673.709179843117</v>
+      </c>
+      <c r="BT6" t="n">
+        <v>1898.452614922407</v>
+      </c>
+      <c r="BU6" t="n">
+        <v>1391.751271143925</v>
+      </c>
+      <c r="BV6" t="n">
+        <v>1555.49256997255</v>
+      </c>
+      <c r="BW6" t="n">
+        <v>1470.140640415737</v>
+      </c>
+      <c r="BX6" t="n">
+        <v>1618.886195773877</v>
+      </c>
+      <c r="BY6" t="n">
+        <v>1438.82437619788</v>
       </c>
     </row>
     <row r="7">
@@ -692,37 +1992,232 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>324.6317986632183</v>
+        <v>712.2876501272201</v>
       </c>
       <c r="C7" t="n">
-        <v>350.1456340418788</v>
+        <v>907.7555898752781</v>
       </c>
       <c r="D7" t="n">
-        <v>370.9677987451415</v>
+        <v>899.415737133525</v>
       </c>
       <c r="E7" t="n">
-        <v>377.6731503940441</v>
+        <v>1620.066104975529</v>
       </c>
       <c r="F7" t="n">
-        <v>353.6707032642191</v>
+        <v>409.4435183511421</v>
       </c>
       <c r="G7" t="n">
-        <v>364.8590157232369</v>
+        <v>478.665042327032</v>
       </c>
       <c r="H7" t="n">
-        <v>339.2015691032469</v>
+        <v>411.748567076176</v>
       </c>
       <c r="I7" t="n">
-        <v>392.5928287176063</v>
+        <v>424.8076508259981</v>
       </c>
       <c r="J7" t="n">
-        <v>387.7875861359022</v>
+        <v>470.727020671435</v>
       </c>
       <c r="K7" t="n">
-        <v>532.1152826546157</v>
+        <v>450.7232738490241</v>
       </c>
       <c r="L7" t="n">
-        <v>486.2243460482219</v>
+        <v>474.0527023047971</v>
+      </c>
+      <c r="M7" t="n">
+        <v>626.452890847641</v>
+      </c>
+      <c r="N7" t="n">
+        <v>630.4970199740851</v>
+      </c>
+      <c r="O7" t="n">
+        <v>611.6755832087121</v>
+      </c>
+      <c r="P7" t="n">
+        <v>684.2520752452881</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>376.9176106373041</v>
+      </c>
+      <c r="R7" t="n">
+        <v>689.6186369993579</v>
+      </c>
+      <c r="S7" t="n">
+        <v>720.433652805405</v>
+      </c>
+      <c r="T7" t="n">
+        <v>664.8991028762611</v>
+      </c>
+      <c r="U7" t="n">
+        <v>776.621375259928</v>
+      </c>
+      <c r="V7" t="n">
+        <v>776.7648332078691</v>
+      </c>
+      <c r="W7" t="n">
+        <v>728.987666750442</v>
+      </c>
+      <c r="X7" t="n">
+        <v>446.007662366497</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>544.379910508962</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>324.486787399214</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>567.3069295648041</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>379.044440547509</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>569.4003721116369</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>639.884285110873</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>728.6802569011461</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>656.760788633675</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>670.1065319708759</v>
+      </c>
+      <c r="AH7" t="n">
+        <v>612.772134210181</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>636.982374490143</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>476.126848074636</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>625.394497241151</v>
+      </c>
+      <c r="AL7" t="n">
+        <v>505.698484358969</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>514.6142165856779</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>671.6311782269211</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>699.7108922387761</v>
+      </c>
+      <c r="AP7" t="n">
+        <v>646.1137827467951</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>533.4806050158311</v>
+      </c>
+      <c r="AR7" t="n">
+        <v>476.902489790331</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>324.219424393084</v>
+      </c>
+      <c r="AT7" t="n">
+        <v>343.837403115888</v>
+      </c>
+      <c r="AU7" t="n">
+        <v>363.4444094310151</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>3150.189533333333</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>1066.247869152084</v>
+      </c>
+      <c r="AX7" t="n">
+        <v>1165.831146022247</v>
+      </c>
+      <c r="AY7" t="n">
+        <v>1015.350537744354</v>
+      </c>
+      <c r="AZ7" t="n">
+        <v>1105.483725819433</v>
+      </c>
+      <c r="BA7" t="n">
+        <v>4797.799119491619</v>
+      </c>
+      <c r="BB7" t="n">
+        <v>3234.263269472807</v>
+      </c>
+      <c r="BC7" t="n">
+        <v>5048.577899838969</v>
+      </c>
+      <c r="BD7" t="n">
+        <v>2554.590607232973</v>
+      </c>
+      <c r="BE7" t="n">
+        <v>4199.959838213883</v>
+      </c>
+      <c r="BF7" t="n">
+        <v>3959.827523860613</v>
+      </c>
+      <c r="BG7" t="n">
+        <v>4378.351747549285</v>
+      </c>
+      <c r="BH7" t="n">
+        <v>4233.177835234814</v>
+      </c>
+      <c r="BI7" t="n">
+        <v>1336</v>
+      </c>
+      <c r="BJ7" t="n">
+        <v>2253.48994962545</v>
+      </c>
+      <c r="BK7" t="n">
+        <v>802.8703</v>
+      </c>
+      <c r="BL7" t="n">
+        <v>997.5</v>
+      </c>
+      <c r="BM7" t="n">
+        <v>834.5</v>
+      </c>
+      <c r="BN7" t="n">
+        <v>1014</v>
+      </c>
+      <c r="BO7" t="n">
+        <v>3088.49679562524</v>
+      </c>
+      <c r="BP7" t="n">
+        <v>2621.81339062411</v>
+      </c>
+      <c r="BQ7" t="n">
+        <v>3897.2607425643</v>
+      </c>
+      <c r="BR7" t="n">
+        <v>4185.50432441001</v>
+      </c>
+      <c r="BS7" t="n">
+        <v>5257.817942003833</v>
+      </c>
+      <c r="BT7" t="n">
+        <v>6092.035543894624</v>
+      </c>
+      <c r="BU7" t="n">
+        <v>4413.418265632176</v>
+      </c>
+      <c r="BV7" t="n">
+        <v>4947.35745394813</v>
+      </c>
+      <c r="BW7" t="n">
+        <v>4699.517335925983</v>
+      </c>
+      <c r="BX7" t="n">
+        <v>4984.982889536515</v>
+      </c>
+      <c r="BY7" t="n">
+        <v>4602.083347639634</v>
       </c>
     </row>
     <row r="8">
@@ -732,37 +2227,232 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2714.763019572504</v>
+        <v>3466.373731147874</v>
       </c>
       <c r="C8" t="n">
-        <v>2936.210470480949</v>
+        <v>4411.674762554062</v>
       </c>
       <c r="D8" t="n">
-        <v>2999.314310180298</v>
+        <v>4518.743718681474</v>
       </c>
       <c r="E8" t="n">
-        <v>3111.551629923011</v>
+        <v>5549.373053125927</v>
       </c>
       <c r="F8" t="n">
-        <v>3002.571606630671</v>
+        <v>2348.513731007125</v>
       </c>
       <c r="G8" t="n">
-        <v>3003.576668248743</v>
+        <v>2791.020711991105</v>
       </c>
       <c r="H8" t="n">
-        <v>2876.622574639217</v>
+        <v>2404.5715041502</v>
       </c>
       <c r="I8" t="n">
-        <v>3230.32160578173</v>
+        <v>2484.190718108605</v>
       </c>
       <c r="J8" t="n">
-        <v>3245.43340987828</v>
+        <v>2662.886714226255</v>
       </c>
       <c r="K8" t="n">
-        <v>3418.42180444752</v>
+        <v>2612.375236091995</v>
       </c>
       <c r="L8" t="n">
-        <v>3241.058766830559</v>
+        <v>2646.53807440495</v>
+      </c>
+      <c r="M8" t="n">
+        <v>3666.157091164975</v>
+      </c>
+      <c r="N8" t="n">
+        <v>3719.930911843795</v>
+      </c>
+      <c r="O8" t="n">
+        <v>3372.427067543215</v>
+      </c>
+      <c r="P8" t="n">
+        <v>3997.622913988991</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>2107.94539919381</v>
+      </c>
+      <c r="R8" t="n">
+        <v>3991.597599254485</v>
+      </c>
+      <c r="S8" t="n">
+        <v>4212.478168900156</v>
+      </c>
+      <c r="T8" t="n">
+        <v>3768.6718179253</v>
+      </c>
+      <c r="U8" t="n">
+        <v>4445.64748534775</v>
+      </c>
+      <c r="V8" t="n">
+        <v>4522.843769262116</v>
+      </c>
+      <c r="W8" t="n">
+        <v>4113.171888843324</v>
+      </c>
+      <c r="X8" t="n">
+        <v>2498.566953207655</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>3215.818705854976</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>1916.923716843795</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>3324.135993063216</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>2253.25550433335</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>3377.82491698234</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>3667.645372110665</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>4365.986547559615</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>3730.977734331485</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>3866.860856773311</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>3571.558782545876</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>3630.414992566505</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>2763.636521657936</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>3483.39701993602</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>2973.50601361462</v>
+      </c>
+      <c r="AM8" t="n">
+        <v>3029.642681192711</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>4051.887410421016</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>4146.83148829323</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>3832.676482595455</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>3212.952900399495</v>
+      </c>
+      <c r="AR8" t="n">
+        <v>2727.68302374458</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>1888.27148433253</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>1983.447830481315</v>
+      </c>
+      <c r="AU8" t="n">
+        <v>2201.31825328723</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>24083.15983333333</v>
+      </c>
+      <c r="AW8" t="n">
+        <v>5070.038360726037</v>
+      </c>
+      <c r="AX8" t="n">
+        <v>5539.523810054163</v>
+      </c>
+      <c r="AY8" t="n">
+        <v>4752.936550856793</v>
+      </c>
+      <c r="AZ8" t="n">
+        <v>5053.534882941815</v>
+      </c>
+      <c r="BA8" t="n">
+        <v>21122.75460713778</v>
+      </c>
+      <c r="BB8" t="n">
+        <v>14363.68096270383</v>
+      </c>
+      <c r="BC8" t="n">
+        <v>22612.36749948912</v>
+      </c>
+      <c r="BD8" t="n">
+        <v>11793.3141094675</v>
+      </c>
+      <c r="BE8" t="n">
+        <v>16260.44543031607</v>
+      </c>
+      <c r="BF8" t="n">
+        <v>15817.18243947031</v>
+      </c>
+      <c r="BG8" t="n">
+        <v>16555.3698080685</v>
+      </c>
+      <c r="BH8" t="n">
+        <v>16063.38397147189</v>
+      </c>
+      <c r="BI8" t="n">
+        <v>5388</v>
+      </c>
+      <c r="BJ8" t="n">
+        <v>6231.9547501924</v>
+      </c>
+      <c r="BK8" t="n">
+        <v>3831.8265</v>
+      </c>
+      <c r="BL8" t="n">
+        <v>4516.25</v>
+      </c>
+      <c r="BM8" t="n">
+        <v>3822.75</v>
+      </c>
+      <c r="BN8" t="n">
+        <v>4701</v>
+      </c>
+      <c r="BO8" t="n">
+        <v>6836.38982943104</v>
+      </c>
+      <c r="BP8" t="n">
+        <v>5354.31353239906</v>
+      </c>
+      <c r="BQ8" t="n">
+        <v>17843.82832670887</v>
+      </c>
+      <c r="BR8" t="n">
+        <v>18154.2537715125</v>
+      </c>
+      <c r="BS8" t="n">
+        <v>21061.78915458805</v>
+      </c>
+      <c r="BT8" t="n">
+        <v>24091.71662989247</v>
+      </c>
+      <c r="BU8" t="n">
+        <v>17285.91237303745</v>
+      </c>
+      <c r="BV8" t="n">
+        <v>19387.33666661473</v>
+      </c>
+      <c r="BW8" t="n">
+        <v>18487.02942640524</v>
+      </c>
+      <c r="BX8" t="n">
+        <v>19323.62305194343</v>
+      </c>
+      <c r="BY8" t="n">
+        <v>17465.30152705693</v>
       </c>
     </row>
     <row r="9">
@@ -772,37 +2462,232 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3441293.778590984</v>
+        <v>8122726.592434363</v>
       </c>
       <c r="C9" t="n">
-        <v>2997519.452074238</v>
+        <v>3086139.294757853</v>
       </c>
       <c r="D9" t="n">
-        <v>3474572.365462308</v>
+        <v>7204266.742329176</v>
       </c>
       <c r="E9" t="n">
-        <v>3766905.59001234</v>
+        <v>2569139.925782104</v>
       </c>
       <c r="F9" t="n">
-        <v>2753403.630072502</v>
+        <v>1698316.65470918</v>
       </c>
       <c r="G9" t="n">
-        <v>2173211.290130805</v>
+        <v>1953657.1430926</v>
       </c>
       <c r="H9" t="n">
-        <v>3039979.376189653</v>
+        <v>2014199.06168294</v>
       </c>
       <c r="I9" t="n">
-        <v>6004868.809911354</v>
+        <v>1790822.73193406</v>
       </c>
       <c r="J9" t="n">
-        <v>2247437.265527637</v>
+        <v>1443755.52817518</v>
       </c>
       <c r="K9" t="n">
-        <v>5375654.536827597</v>
+        <v>1564591.58663698</v>
       </c>
       <c r="L9" t="n">
-        <v>4239740.357313359</v>
+        <v>1970313.74127984</v>
+      </c>
+      <c r="M9" t="n">
+        <v>2470661.90715718</v>
+      </c>
+      <c r="N9" t="n">
+        <v>2527283.75416462</v>
+      </c>
+      <c r="O9" t="n">
+        <v>2105847.42581576</v>
+      </c>
+      <c r="P9" t="n">
+        <v>2421202.90838998</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>1466816.39147648</v>
+      </c>
+      <c r="R9" t="n">
+        <v>2861788.170666261</v>
+      </c>
+      <c r="S9" t="n">
+        <v>2785112.37681754</v>
+      </c>
+      <c r="T9" t="n">
+        <v>5038810.982452061</v>
+      </c>
+      <c r="U9" t="n">
+        <v>5636538.305159081</v>
+      </c>
+      <c r="V9" t="n">
+        <v>6049808.34863592</v>
+      </c>
+      <c r="W9" t="n">
+        <v>3456150.8082959</v>
+      </c>
+      <c r="X9" t="n">
+        <v>1599383.84789106</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>2408499.85809554</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>1153911.62847246</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>1847383.16277328</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>1924986.18972528</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>1963689.22389178</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>2583918.8280532</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>3856207.218654341</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>2799825.38531674</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>3081100.34485264</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>2326375.29938</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>1977546.07586316</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>2151719.3254238</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>3293436.0035962</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>1824004.88094594</v>
+      </c>
+      <c r="AM9" t="n">
+        <v>2693794.69019408</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>2287799.90739608</v>
+      </c>
+      <c r="AO9" t="n">
+        <v>3008709.25558984</v>
+      </c>
+      <c r="AP9" t="n">
+        <v>2736623.22405714</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>3265940.9522993</v>
+      </c>
+      <c r="AR9" t="n">
+        <v>2398317.22903388</v>
+      </c>
+      <c r="AS9" t="n">
+        <v>1673813.56260536</v>
+      </c>
+      <c r="AT9" t="n">
+        <v>1671361.1306579</v>
+      </c>
+      <c r="AU9" t="n">
+        <v>1447457.46153008</v>
+      </c>
+      <c r="AV9" t="n">
+        <v>2040565.936933333</v>
+      </c>
+      <c r="AW9" t="n">
+        <v>2650588.786217585</v>
+      </c>
+      <c r="AX9" t="n">
+        <v>2980879.128088631</v>
+      </c>
+      <c r="AY9" t="n">
+        <v>5498558.33502333</v>
+      </c>
+      <c r="AZ9" t="n">
+        <v>5568349.405127079</v>
+      </c>
+      <c r="BA9" t="n">
+        <v>3672230.851263796</v>
+      </c>
+      <c r="BB9" t="n">
+        <v>2530817.22048714</v>
+      </c>
+      <c r="BC9" t="n">
+        <v>3841111.080042755</v>
+      </c>
+      <c r="BD9" t="n">
+        <v>2055972.214523255</v>
+      </c>
+      <c r="BE9" t="n">
+        <v>2325577.519082672</v>
+      </c>
+      <c r="BF9" t="n">
+        <v>2181179.000166196</v>
+      </c>
+      <c r="BG9" t="n">
+        <v>2348400.968177486</v>
+      </c>
+      <c r="BH9" t="n">
+        <v>2267621.734259108</v>
+      </c>
+      <c r="BI9" t="n">
+        <v>1643440</v>
+      </c>
+      <c r="BJ9" t="n">
+        <v>1589836.91145789</v>
+      </c>
+      <c r="BK9" t="n">
+        <v>1575311</v>
+      </c>
+      <c r="BL9" t="n">
+        <v>1276423</v>
+      </c>
+      <c r="BM9" t="n">
+        <v>816687</v>
+      </c>
+      <c r="BN9" t="n">
+        <v>1270793</v>
+      </c>
+      <c r="BO9" t="n">
+        <v>1392598.80028636</v>
+      </c>
+      <c r="BP9" t="n">
+        <v>746357.568074079</v>
+      </c>
+      <c r="BQ9" t="n">
+        <v>3989325.64061538</v>
+      </c>
+      <c r="BR9" t="n">
+        <v>3563066.28214841</v>
+      </c>
+      <c r="BS9" t="n">
+        <v>2186908.808510384</v>
+      </c>
+      <c r="BT9" t="n">
+        <v>1465364.870438074</v>
+      </c>
+      <c r="BU9" t="n">
+        <v>1073011.442711933</v>
+      </c>
+      <c r="BV9" t="n">
+        <v>1145706.187841673</v>
+      </c>
+      <c r="BW9" t="n">
+        <v>1027047.573270711</v>
+      </c>
+      <c r="BX9" t="n">
+        <v>1107606.637430847</v>
+      </c>
+      <c r="BY9" t="n">
+        <v>1026338.674711787</v>
       </c>
     </row>
   </sheetData>

</xml_diff>